<commit_message>
Deployed 0f3fefc88 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/issues_list.xlsx
+++ b/main/issues_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C42"/>
+  <dimension ref="A1:C45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -584,12 +584,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
+          <t>0f19ac6e-dc86-445b-b2da-7b61a389222e</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
+          <t>Broken link (404): http://www.env.gov.bc.ca/omfd/reports/Kelp2007-HakaiPass.pdf</t>
         </is>
       </c>
     </row>
@@ -599,12 +599,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0f19ac6e-dc86-445b-b2da-7b61a389222e</t>
+          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Broken link (404): http://www.env.gov.bc.ca/omfd/reports/Kelp2007-HakaiPass.pdf</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -644,12 +644,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
+          <t>2709d7b1-22e1-4268-bcda-dc0c79f2878e</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
+          <t>Invalid Resource URL: https://doi.org/10.5281/zenodo.4005400 returned status_code=504</t>
         </is>
       </c>
     </row>
@@ -674,12 +674,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
+          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-qu5-mooring-data</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -689,18 +689,18 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Metadata mismatch: publication year CKAN='2026' | DataCite='2020'</t>
+          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-qu5-mooring-data</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -709,13 +709,13 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Metadata mismatch: publication year CKAN='2026' | DataCite='2020'</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -724,22 +724,22 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>d3ed88cb-4f38-4c2e-a966-3dd49c9cafec</t>
+          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.1016/j.ecss.2020.107103' in CKAN not found in DataCite</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -749,12 +749,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>c5e60545-c6f2-4945-af0a-21812ba5f0d9</t>
+          <t>d3ed88cb-4f38-4c2e-a966-3dd49c9cafec</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Broken link (202): https://jakelawlor.shinyapps.io/optimize_ProdVersion/</t>
+          <t>Metadata mismatch: related work '10.1016/j.ecss.2020.107103' in CKAN not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -764,12 +764,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
+          <t>c5e60545-c6f2-4945-af0a-21812ba5f0d9</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
+          <t>Broken link (202): https://jakelawlor.shinyapps.io/optimize_ProdVersion/</t>
         </is>
       </c>
     </row>
@@ -779,27 +779,27 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>bc1133da-5601-4f92-bc53-41be547c936b</t>
+          <t>d70bcd3d-dc07-479f-856f-ad70d11c51f1</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Invalid Resource URL: https://zenodo.org/uploads/15344675 returned status_code=504</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>bc1133da-5601-4f92-bc53-41be547c936b</t>
+          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -809,12 +809,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>bc1133da-5601-4f92-bc53-41be547c936b</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -824,12 +824,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>bc1133da-5601-4f92-bc53-41be547c936b</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -844,7 +844,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
         </is>
       </c>
     </row>
@@ -859,7 +859,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
         </is>
       </c>
     </row>
@@ -869,42 +869,42 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>c7a168e8-f15e-446f-a49d-0b4a1f043ac2</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Broken link (202): https://fjedna.shinyapps.io/census-app1/</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>c1e0447b-a06c-44c8-abd0-3108b2f00b7a</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>c1e0447b-a06c-44c8-abd0-3108b2f00b7a</t>
+          <t>c7a168e8-f15e-446f-a49d-0b4a1f043ac2</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Broken link (202): https://fjedna.shinyapps.io/census-app1/</t>
         </is>
       </c>
     </row>
@@ -914,12 +914,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>b7638e0b-e734-4a96-97af-9e7729b61831</t>
+          <t>c1e0447b-a06c-44c8-abd0-3108b2f00b7a</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Tentative dataset should not have a version</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -929,12 +929,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>b7638e0b-e734-4a96-97af-9e7729b61831</t>
+          <t>c1e0447b-a06c-44c8-abd0-3108b2f00b7a</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -944,42 +944,42 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>613ba2f9-b21d-445f-8eaa-f42950c9350b</t>
+          <t>b7638e0b-e734-4a96-97af-9e7729b61831</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf returned status_code=404</t>
+          <t>Tentative dataset should not have a version</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>39818579-9692-4256-9810-d8b80e9821aa</t>
+          <t>b7638e0b-e734-4a96-97af-9e7729b61831</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>39818579-9692-4256-9810-d8b80e9821aa</t>
+          <t>613ba2f9-b21d-445f-8eaa-f42950c9350b</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -989,12 +989,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>39818579-9692-4256-9810-d8b80e9821aa</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
@@ -1004,12 +1004,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>39818579-9692-4256-9810-d8b80e9821aa</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -1019,25 +1019,70 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>3fbbd892-55cd-4c96-9669-cecefe726b3f</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.1016/j.pocean.2022.102843' in CKAN not found in DataCite</t>
+          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>0</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>3fbbd892-55cd-4c96-9669-cecefe726b3f</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Metadata mismatch: related work '10.1016/j.pocean.2022.102843' in CKAN not found in DataCite</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>0</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>b01f58f7-1518-4829-aff6-ac4a8f2c0616</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Broken link (404): https://hakai-segmentation.readthedocs.io/en/latest/</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>0</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
           <t>acd6c43f-6cbd-43c8-9bff-7d9ae6630295</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C45" t="inlineStr">
         <is>
           <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf returned status_code=404</t>
         </is>

</xml_diff>

<commit_message>
Deployed b19bb2f4e to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/issues_list.xlsx
+++ b/main/issues_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C62"/>
+  <dimension ref="A1:C48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -434,33 +434,33 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
+          <t>97677e6b-1d06-4466-8849-043df22984c1</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Broken link (404): http://geobc.gov.bc.ca/base-mapping/atlas/trim/</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>97677e6b-1d06-4466-8849-043df22984c1</t>
+          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Broken link (404): http://geobc.gov.bc.ca/base-mapping/atlas/trim/</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -475,266 +475,266 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>52d607c9-46cd-4be9-a752-1b5446272f32</t>
+          <t>646dd927-3248-4fc9-970c-abea15f7d304</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>52d607c9-46cd-4be9-a752-1b5446272f32</t>
+          <t>646dd927-3248-4fc9-970c-abea15f7d304</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>646dd927-3248-4fc9-970c-abea15f7d304</t>
+          <t>44bdc298-1329-400a-bc02-4d35d251865d</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: related identifier 'dx.doi.org/10.17504/protocols.io.eq2lywxwpvx9/v1' (IsSupplementedBy) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>646dd927-3248-4fc9-970c-abea15f7d304</t>
+          <t>bd461764-55b0-4c63-935a-5e9d1d5a6fed</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-itracksept2023 returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>44bdc298-1329-400a-bc02-4d35d251865d</t>
+          <t>2de5b0d2-71b1-4041-bd01-118e9c529dac</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'dx.doi.org/10.17504/protocols.io.eq2lywxwpvx9/v1' (IsSupplementedBy) in DataCite not found in CKAN</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>bd461764-55b0-4c63-935a-5e9d1d5a6fed</t>
+          <t>da040f55-984d-490d-b917-a67856de4bac</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-itracksept2023 returned status_code=404</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-seastars2024 returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2de5b0d2-71b1-4041-bd01-118e9c529dac</t>
+          <t>0ce3ee5b-425b-4eb0-a201-96bdfb795a3f</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Tentative dataset should not have a version</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2de5b0d2-71b1-4041-bd01-118e9c529dac</t>
+          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>da040f55-984d-490d-b917-a67856de4bac</t>
+          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-seastars2024 returned status_code=404</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>0ce3ee5b-425b-4eb0-a201-96bdfb795a3f</t>
+          <t>0f19ac6e-dc86-445b-b2da-7b61a389222e</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Broken link (404): http://www.env.gov.bc.ca/omfd/reports/Kelp2007-HakaiPass.pdf</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
+          <t>c4932b55-1dd8-4f2f-89da-5822056ecc37</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
+          <t>Broken link (404): https://doi.org/10.21966/ekwk-r335</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
+          <t>1a2aa5c8-9a83-46f7-967d-1127436c2084</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>0f19ac6e-dc86-445b-b2da-7b61a389222e</t>
+          <t>13dc3c6c-9dd4-47a4-92ad-681c653d3565</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Broken link (404): http://www.env.gov.bc.ca/omfd/reports/Kelp2007-HakaiPass.pdf</t>
+          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>4b04cbfe-71f4-47b4-b028-3fcd24e7cff2</t>
+          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Jenn Burt' in DataCite not found in CKAN record</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>4b04cbfe-71f4-47b4-b028-3fcd24e7cff2</t>
+          <t>33bb67af-4d61-4b15-93a9-f3ab2498430b</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'J. Burt' in CKAN record not found in DataCite</t>
+          <t>Broken link (404): http://www.env.gov.bc.ca/omfd/reports/Kelp2007-HakaiPass.pdf</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>4b04cbfe-71f4-47b4-b028-3fcd24e7cff2</t>
+          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.25607/OBP-2068' (IsSupplementedBy) in DataCite not found in CKAN</t>
+          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-qu5-mooring-data</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>c4932b55-1dd8-4f2f-89da-5822056ecc37</t>
+          <t>c035b81c-0fc3-446e-bec5-8b8933ae874b</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Broken link (404): https://doi.org/10.21966/ekwk-r335</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>1a2aa5c8-9a83-46f7-967d-1127436c2084</t>
+          <t>ddf1f914-89b7-41fe-8e72-e5217476fc09</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -745,131 +745,131 @@
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>13dc3c6c-9dd4-47a4-92ad-681c653d3565</t>
+          <t>c5e60545-c6f2-4945-af0a-21812ba5f0d9</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf</t>
+          <t>Broken link (202): https://jakelawlor.shinyapps.io/optimize_ProdVersion/</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>33bb67af-4d61-4b15-93a9-f3ab2498430b</t>
+          <t>5216f7f5-a569-4f76-9cab-171f1e847498</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Broken link (404): http://www.env.gov.bc.ca/omfd/reports/Kelp2007-HakaiPass.pdf</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
+          <t>1f4b5991-bbcb-416b-807c-ed8ca5f4d9f4</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
+          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-qu5-mooring-data</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Metadata mismatch: publication year CKAN='2026' | DataCite='2020'</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>2</v>
+        <v>27</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>c035b81c-0fc3-446e-bec5-8b8933ae874b</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>ddf1f914-89b7-41fe-8e72-e5217476fc09</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -880,71 +880,71 @@
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>d3ed88cb-4f38-4c2e-a966-3dd49c9cafec</t>
+          <t>1af6a43a-e73b-4774-8e10-b9f2928ab133</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related work '10.1016/j.ecss.2020.107103' in CKAN not found in DataCite</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>c5e60545-c6f2-4945-af0a-21812ba5f0d9</t>
+          <t>c1e0447b-a06c-44c8-abd0-3108b2f00b7a</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Broken link (202): https://jakelawlor.shinyapps.io/optimize_ProdVersion/</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>5216f7f5-a569-4f76-9cab-171f1e847498</t>
+          <t>c1e0447b-a06c-44c8-abd0-3108b2f00b7a</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
+          <t>c7a168e8-f15e-446f-a49d-0b4a1f043ac2</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
+          <t>Broken link (202): https://fjedna.shinyapps.io/census-app1/</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>1f4b5991-bbcb-416b-807c-ed8ca5f4d9f4</t>
+          <t>d320d90e-96bf-4993-81c5-f1f57886b0e6</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -955,101 +955,101 @@
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
+          <t>613ba2f9-b21d-445f-8eaa-f42950c9350b</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>bc1133da-5601-4f92-bc53-41be547c936b</t>
+          <t>b7638e0b-e734-4a96-97af-9e7729b61831</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>1</v>
+        <v>37</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>bc1133da-5601-4f92-bc53-41be547c936b</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>1</v>
+        <v>39</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>879a98f9-7e86-46dc-9449-e05cbf720b1e</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>4c7b7347-767d-45e4-b3ad-7e0133b31e1c</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>1</v>
+        <v>41</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>8dadb6a8-8eb2-44ea-9d2d-c4332e4c544b</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1060,11 +1060,11 @@
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>1af6a43a-e73b-4774-8e10-b9f2928ab133</t>
+          <t>35245eae-e508-47da-bcf7-54346cda086a</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1075,271 +1075,61 @@
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>0</v>
+        <v>43</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>c7a168e8-f15e-446f-a49d-0b4a1f043ac2</t>
+          <t>5177d019-598e-4415-b778-9688403652c8</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Broken link (202): https://fjedna.shinyapps.io/census-app1/</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>0</v>
+        <v>44</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>c1e0447b-a06c-44c8-abd0-3108b2f00b7a</t>
+          <t>b01f58f7-1518-4829-aff6-ac4a8f2c0616</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Broken link (404): https://hakai-segmentation.readthedocs.io/en/latest/</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>1</v>
+        <v>45</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>c1e0447b-a06c-44c8-abd0-3108b2f00b7a</t>
+          <t>acd6c43f-6cbd-43c8-9bff-7d9ae6630295</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>0</v>
+        <v>46</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>d320d90e-96bf-4993-81c5-f1f57886b0e6</t>
+          <t>5576c279-6d3a-4323-8104-0e1040d9906c</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>No funder</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="n">
-        <v>0</v>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>613ba2f9-b21d-445f-8eaa-f42950c9350b</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf returned status_code=404</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="n">
-        <v>0</v>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>b7638e0b-e734-4a96-97af-9e7729b61831</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>No funder</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="n">
-        <v>0</v>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>39818579-9692-4256-9810-d8b80e9821aa</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="n">
-        <v>1</v>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>39818579-9692-4256-9810-d8b80e9821aa</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="n">
-        <v>0</v>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="n">
-        <v>1</v>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="n">
-        <v>0</v>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>879a98f9-7e86-46dc-9449-e05cbf720b1e</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>No funder</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="n">
-        <v>0</v>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>4c7b7347-767d-45e4-b3ad-7e0133b31e1c</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>No funder</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="n">
-        <v>0</v>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>8dadb6a8-8eb2-44ea-9d2d-c4332e4c544b</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>No funder</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="n">
-        <v>0</v>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>35245eae-e508-47da-bcf7-54346cda086a</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>No funder</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="n">
-        <v>0</v>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>5177d019-598e-4415-b778-9688403652c8</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>No funder</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="n">
-        <v>0</v>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>3fbbd892-55cd-4c96-9669-cecefe726b3f</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: related work '10.1016/j.pocean.2022.102843' in CKAN not found in DataCite</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="n">
-        <v>0</v>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>b01f58f7-1518-4829-aff6-ac4a8f2c0616</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>Broken link (404): https://hakai-segmentation.readthedocs.io/en/latest/</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="n">
-        <v>0</v>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>acd6c43f-6cbd-43c8-9bff-7d9ae6630295</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf returned status_code=404</t>
+          <t>Contact missing affiliation: Okamoto, Daniel</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deployed 81c041b89 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/issues_list.xlsx
+++ b/main/issues_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C34"/>
+  <dimension ref="A1:C44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -445,7 +445,7 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -460,7 +460,7 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -475,97 +475,97 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>44bdc298-1329-400a-bc02-4d35d251865d</t>
+          <t>bd461764-55b0-4c63-935a-5e9d1d5a6fed</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'dx.doi.org/10.17504/protocols.io.eq2lywxwpvx9/v1' (IsSupplementedBy) in DataCite not found in CKAN</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-itracksept2023 returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>bd461764-55b0-4c63-935a-5e9d1d5a6fed</t>
+          <t>da040f55-984d-490d-b917-a67856de4bac</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-itracksept2023 returned status_code=404</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-seastars2024 returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>da040f55-984d-490d-b917-a67856de4bac</t>
+          <t>5fc21b4d-2dfa-4908-8aaf-90a82509324a</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-seastars2024 returned status_code=404</t>
+          <t>Metadata mismatch: creator 'Dalhousie College' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
+          <t>5fc21b4d-2dfa-4908-8aaf-90a82509324a</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
+          <t>Metadata mismatch: author 'Whale Ecology &amp; Conservation Lab' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
+          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
+          <t>0f19ac6e-dc86-445b-b2da-7b61a389222e</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Broken link (404): http://www.env.gov.bc.ca/omfd/reports/Kelp2007-HakaiPass.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -580,37 +580,37 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0f19ac6e-dc86-445b-b2da-7b61a389222e</t>
+          <t>37440dfd-53f8-462b-a544-b6c8d39c44cd</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Broken link (404): http://www.env.gov.bc.ca/omfd/reports/Kelp2007-HakaiPass.pdf</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>1bba6c8a-b99c-4fbd-8eae-7c8b771a841d</t>
+          <t>37440dfd-53f8-462b-a544-b6c8d39c44cd</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Broken link (500): https://www.pmel.noaa.gov/co2/story/2016+West+Coast+Ocean+Acidification+Cruise</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -625,7 +625,7 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -640,7 +640,7 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -655,7 +655,7 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -670,7 +670,7 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -685,7 +685,7 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -700,7 +700,7 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -715,211 +715,361 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
+          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>c1e0447b-a06c-44c8-abd0-3108b2f00b7a</t>
+          <t>6c99bd67-3be1-4818-bf01-dfa56e910db3</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>c1e0447b-a06c-44c8-abd0-3108b2f00b7a</t>
+          <t>6c99bd67-3be1-4818-bf01-dfa56e910db3</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>c7a168e8-f15e-446f-a49d-0b4a1f043ac2</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Broken link (202): https://fjedna.shinyapps.io/census-app1/</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>613ba2f9-b21d-445f-8eaa-f42950c9350b</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf returned status_code=404</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>c1e0447b-a06c-44c8-abd0-3108b2f00b7a</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>29</v>
+        <v>1</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>c1e0447b-a06c-44c8-abd0-3108b2f00b7a</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>b01f58f7-1518-4829-aff6-ac4a8f2c0616</t>
+          <t>0074861a-39f2-42c1-ae71-abef4f78fd78</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Broken link (404): https://hakai-segmentation.readthedocs.io/en/latest/</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>31</v>
+        <v>1</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>acd6c43f-6cbd-43c8-9bff-7d9ae6630295</t>
+          <t>0074861a-39f2-42c1-ae71-abef4f78fd78</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf returned status_code=404</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>5576c279-6d3a-4323-8104-0e1040d9906c</t>
+          <t>c7a168e8-f15e-446f-a49d-0b4a1f043ac2</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Contact missing affiliation: Okamoto, Daniel</t>
+          <t>Broken link (202): https://fjedna.shinyapps.io/census-app1/</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>0</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>613ba2f9-b21d-445f-8eaa-f42950c9350b</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf returned status_code=404</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>0</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>9eda1bfc-0d13-4e1d-9542-b9a7cce16991</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>1</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>9eda1bfc-0d13-4e1d-9542-b9a7cce16991</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>0</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>39818579-9692-4256-9810-d8b80e9821aa</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>1</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>39818579-9692-4256-9810-d8b80e9821aa</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>0</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>1</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>0</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>b01f58f7-1518-4829-aff6-ac4a8f2c0616</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Broken link (404): https://hakai-segmentation.readthedocs.io/en/latest/</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>0</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>acd6c43f-6cbd-43c8-9bff-7d9ae6630295</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf returned status_code=404</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>0</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>58d56d16-6350-4b01-a062-6bdb2d9f89b4</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Invalid Resource URL: https://www.ncei.noaa.gov/data/oceans/ncei/ocads/data/0276518/ returned status_code=502</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deployed adca83bc8 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/issues_list.xlsx
+++ b/main/issues_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C44"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -509,27 +509,27 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>5fc21b4d-2dfa-4908-8aaf-90a82509324a</t>
+          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Dalhousie College' in DataCite not found in CKAN record</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>5fc21b4d-2dfa-4908-8aaf-90a82509324a</t>
+          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Whale Ecology &amp; Conservation Lab' in CKAN record not found in DataCite</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -539,12 +539,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
+          <t>0f19ac6e-dc86-445b-b2da-7b61a389222e</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
+          <t>Broken link (404): http://www.env.gov.bc.ca/omfd/reports/Kelp2007-HakaiPass.pdf</t>
         </is>
       </c>
     </row>
@@ -554,12 +554,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0f19ac6e-dc86-445b-b2da-7b61a389222e</t>
+          <t>c4932b55-1dd8-4f2f-89da-5822056ecc37</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Broken link (404): http://www.env.gov.bc.ca/omfd/reports/Kelp2007-HakaiPass.pdf</t>
+          <t>Broken link (404): https://doi.org/10.21966/ekwk-r335</t>
         </is>
       </c>
     </row>
@@ -569,12 +569,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
+          <t>13dc3c6c-9dd4-47a4-92ad-681c653d3565</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
+          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf</t>
         </is>
       </c>
     </row>
@@ -584,27 +584,27 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>37440dfd-53f8-462b-a544-b6c8d39c44cd</t>
+          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>37440dfd-53f8-462b-a544-b6c8d39c44cd</t>
+          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-qu5-mooring-data</t>
         </is>
       </c>
     </row>
@@ -614,12 +614,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>c4932b55-1dd8-4f2f-89da-5822056ecc37</t>
+          <t>33bb67af-4d61-4b15-93a9-f3ab2498430b</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Broken link (404): https://doi.org/10.21966/ekwk-r335</t>
+          <t>Broken link (404): http://www.env.gov.bc.ca/omfd/reports/Kelp2007-HakaiPass.pdf</t>
         </is>
       </c>
     </row>
@@ -629,12 +629,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>13dc3c6c-9dd4-47a4-92ad-681c653d3565</t>
+          <t>c5e60545-c6f2-4945-af0a-21812ba5f0d9</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf</t>
+          <t>Broken link (202): https://jakelawlor.shinyapps.io/optimize_ProdVersion/</t>
         </is>
       </c>
     </row>
@@ -644,12 +644,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
+          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -659,12 +659,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>33bb67af-4d61-4b15-93a9-f3ab2498430b</t>
+          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Broken link (404): http://www.env.gov.bc.ca/omfd/reports/Kelp2007-HakaiPass.pdf</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -674,27 +674,27 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-qu5-mooring-data</t>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>c5e60545-c6f2-4945-af0a-21812ba5f0d9</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Broken link (202): https://jakelawlor.shinyapps.io/optimize_ProdVersion/</t>
+          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
         </is>
       </c>
     </row>
@@ -704,42 +704,42 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2916abf5-419e-4cd7-8e25-f45f07a21313</t>
+          <t>c7a168e8-f15e-446f-a49d-0b4a1f043ac2</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Broken link (202): https://fjedna.shinyapps.io/census-app1/</t>
         </is>
       </c>
     </row>
@@ -749,42 +749,42 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
+          <t>c1e0447b-a06c-44c8-abd0-3108b2f00b7a</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>c1e0447b-a06c-44c8-abd0-3108b2f00b7a</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>613ba2f9-b21d-445f-8eaa-f42950c9350b</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -794,12 +794,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>6c99bd67-3be1-4818-bf01-dfa56e910db3</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
         </is>
       </c>
     </row>
@@ -809,12 +809,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>6c99bd67-3be1-4818-bf01-dfa56e910db3</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
         </is>
       </c>
     </row>
@@ -824,27 +824,27 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>b01f58f7-1518-4829-aff6-ac4a8f2c0616</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Broken link (404): https://hakai-segmentation.readthedocs.io/en/latest/</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>acd6c43f-6cbd-43c8-9bff-7d9ae6630295</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -854,220 +854,10 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>c1e0447b-a06c-44c8-abd0-3108b2f00b7a</t>
+          <t>58d56d16-6350-4b01-a062-6bdb2d9f89b4</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
-        <is>
-          <t>No version</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="n">
-        <v>1</v>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>c1e0447b-a06c-44c8-abd0-3108b2f00b7a</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>No DOI defined</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="n">
-        <v>0</v>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>0074861a-39f2-42c1-ae71-abef4f78fd78</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="n">
-        <v>1</v>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>0074861a-39f2-42c1-ae71-abef4f78fd78</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="n">
-        <v>0</v>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>c7a168e8-f15e-446f-a49d-0b4a1f043ac2</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>Broken link (202): https://fjedna.shinyapps.io/census-app1/</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="n">
-        <v>0</v>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>613ba2f9-b21d-445f-8eaa-f42950c9350b</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf returned status_code=404</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="n">
-        <v>0</v>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>9eda1bfc-0d13-4e1d-9542-b9a7cce16991</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="n">
-        <v>1</v>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>9eda1bfc-0d13-4e1d-9542-b9a7cce16991</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="n">
-        <v>0</v>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>39818579-9692-4256-9810-d8b80e9821aa</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="n">
-        <v>1</v>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>39818579-9692-4256-9810-d8b80e9821aa</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="n">
-        <v>0</v>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="n">
-        <v>1</v>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="n">
-        <v>0</v>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>b01f58f7-1518-4829-aff6-ac4a8f2c0616</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>Broken link (404): https://hakai-segmentation.readthedocs.io/en/latest/</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="n">
-        <v>0</v>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>acd6c43f-6cbd-43c8-9bff-7d9ae6630295</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf returned status_code=404</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="n">
-        <v>0</v>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>58d56d16-6350-4b01-a062-6bdb2d9f89b4</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
         <is>
           <t>Invalid Resource URL: https://www.ncei.noaa.gov/data/oceans/ncei/ocads/data/0276518/ returned status_code=502</t>
         </is>

</xml_diff>

<commit_message>
Deployed a4203cfd1 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/issues_list.xlsx
+++ b/main/issues_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -439,52 +439,52 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Broken link (404): http://geobc.gov.bc.ca/base-mapping/atlas/trim/</t>
+          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>646dd927-3248-4fc9-970c-abea15f7d304</t>
+          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Metadata mismatch: creator 'Government of British Columbia' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>646dd927-3248-4fc9-970c-abea15f7d304</t>
+          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>bd461764-55b0-4c63-935a-5e9d1d5a6fed</t>
+          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-itracksept2023 returned status_code=404</t>
+          <t>Metadata mismatch: author 'GeoBC Branch' in CKAN record not found in DataCite</t>
         </is>
       </c>
     </row>
@@ -494,27 +494,27 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>da040f55-984d-490d-b917-a67856de4bac</t>
+          <t>646dd927-3248-4fc9-970c-abea15f7d304</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-seastars2024 returned status_code=404</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
+          <t>646dd927-3248-4fc9-970c-abea15f7d304</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -524,12 +524,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0f19ac6e-dc86-445b-b2da-7b61a389222e</t>
+          <t>bd461764-55b0-4c63-935a-5e9d1d5a6fed</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Broken link (404): http://www.env.gov.bc.ca/omfd/reports/Kelp2007-HakaiPass.pdf</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-itracksept2023 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -539,12 +539,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
+          <t>da040f55-984d-490d-b917-a67856de4bac</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-seastars2024 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -554,12 +554,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>c4932b55-1dd8-4f2f-89da-5822056ecc37</t>
+          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Broken link (404): https://doi.org/10.21966/ekwk-r335</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -569,12 +569,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>13dc3c6c-9dd4-47a4-92ad-681c653d3565</t>
+          <t>1bba6c8a-b99c-4fbd-8eae-7c8b771a841d</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf</t>
+          <t>Broken link (500): https://www.pmel.noaa.gov/co2/story/2016+West+Coast+Ocean+Acidification+Cruise</t>
         </is>
       </c>
     </row>
@@ -584,12 +584,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
+          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -599,12 +599,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
+          <t>c4932b55-1dd8-4f2f-89da-5822056ecc37</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-qu5-mooring-data</t>
+          <t>Broken link (404): https://doi.org/10.21966/ekwk-r335</t>
         </is>
       </c>
     </row>
@@ -629,12 +629,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
+          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -644,12 +644,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
+          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
+          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-qu5-mooring-data</t>
         </is>
       </c>
     </row>
@@ -659,27 +659,27 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -689,33 +689,33 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>c5e60545-c6f2-4945-af0a-21812ba5f0d9</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Broken link (202): https://jakelawlor.shinyapps.io/optimize_ProdVersion/</t>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -724,37 +724,37 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>c1e0447b-a06c-44c8-abd0-3108b2f00b7a</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>c1e0447b-a06c-44c8-abd0-3108b2f00b7a</t>
+          <t>c7a168e8-f15e-446f-a49d-0b4a1f043ac2</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Broken link (202): https://fjedna.shinyapps.io/census-app1/</t>
         </is>
       </c>
     </row>
@@ -764,27 +764,27 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>c7a168e8-f15e-446f-a49d-0b4a1f043ac2</t>
+          <t>c1e0447b-a06c-44c8-abd0-3108b2f00b7a</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Broken link (202): https://fjedna.shinyapps.io/census-app1/</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>613ba2f9-b21d-445f-8eaa-f42950c9350b</t>
+          <t>c1e0447b-a06c-44c8-abd0-3108b2f00b7a</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf returned status_code=404</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -815,36 +815,6 @@
       <c r="C27" t="inlineStr">
         <is>
           <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="n">
-        <v>0</v>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>b01f58f7-1518-4829-aff6-ac4a8f2c0616</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>Broken link (404): https://hakai-segmentation.readthedocs.io/en/latest/</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="n">
-        <v>0</v>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>acd6c43f-6cbd-43c8-9bff-7d9ae6630295</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-datasets/raw/development/datasets_documents/HakaiWaterPropertiesProfiles/Hakai_Water_Properties_Processing_and_QAQC_Procedure_20210331.pdf returned status_code=404</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deployed 791d0b550 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/issues_list.xlsx
+++ b/main/issues_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -539,12 +539,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>da040f55-984d-490d-b917-a67856de4bac</t>
+          <t>52d607c9-46cd-4be9-a752-1b5446272f32</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-seastars2024 returned status_code=404</t>
+          <t>Broken link (500): https://drive.google.com/file/d/1SXXmpGLEPS6wgxvcZXvnENneqFk5KuvJ/view?usp=drive_link</t>
         </is>
       </c>
     </row>
@@ -554,12 +554,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
+          <t>da040f55-984d-490d-b917-a67856de4bac</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-seastars2024 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -569,12 +569,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>1bba6c8a-b99c-4fbd-8eae-7c8b771a841d</t>
+          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Broken link (500): https://www.pmel.noaa.gov/co2/story/2016+West+Coast+Ocean+Acidification+Cruise</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -694,7 +694,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
         </is>
       </c>
     </row>
@@ -709,7 +709,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
         </is>
       </c>
     </row>
@@ -749,12 +749,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>c7a168e8-f15e-446f-a49d-0b4a1f043ac2</t>
+          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Broken link (202): https://fjedna.shinyapps.io/census-app1/</t>
+          <t>Broken link (connection error): https://www2.gov.bc.ca/gov/content/data/geographic-data-services/topographic-data/freshwater</t>
         </is>
       </c>
     </row>
@@ -764,27 +764,27 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>c1e0447b-a06c-44c8-abd0-3108b2f00b7a</t>
+          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>No version</t>
+          <t>Invalid Resource URL: https://drive.google.com/file/d/1GWVbbZg0UM-0GLQA9urqg4uySDrLPr6D/view?usp=sharing returned status_code=500</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>c1e0447b-a06c-44c8-abd0-3108b2f00b7a</t>
+          <t>c7a168e8-f15e-446f-a49d-0b4a1f043ac2</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Broken link (202): https://fjedna.shinyapps.io/census-app1/</t>
         </is>
       </c>
     </row>
@@ -794,12 +794,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>c1e0447b-a06c-44c8-abd0-3108b2f00b7a</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -809,12 +809,42 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
+          <t>c1e0447b-a06c-44c8-abd0-3108b2f00b7a</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>No DOI defined</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>0</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
           <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>1</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deployed 7a3f0f37b to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/issues_list.xlsx
+++ b/main/issues_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -539,12 +539,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>52d607c9-46cd-4be9-a752-1b5446272f32</t>
+          <t>da040f55-984d-490d-b917-a67856de4bac</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Broken link (500): https://drive.google.com/file/d/1SXXmpGLEPS6wgxvcZXvnENneqFk5KuvJ/view?usp=drive_link</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-seastars2024 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -554,12 +554,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>da040f55-984d-490d-b917-a67856de4bac</t>
+          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-seastars2024 returned status_code=404</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -569,12 +569,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
+          <t>432b05ce-8904-4094-94bf-b97fb6636e41</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
+          <t>Record DOI HTTPS link is failling: https://doi.org/10.21966/kp87-sf64 status_code=502</t>
         </is>
       </c>
     </row>
@@ -614,12 +614,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>33bb67af-4d61-4b15-93a9-f3ab2498430b</t>
+          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Broken link (404): http://www.env.gov.bc.ca/omfd/reports/Kelp2007-HakaiPass.pdf</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -629,12 +629,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
+          <t>33bb67af-4d61-4b15-93a9-f3ab2498430b</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
+          <t>Broken link (404): http://www.env.gov.bc.ca/omfd/reports/Kelp2007-HakaiPass.pdf</t>
         </is>
       </c>
     </row>
@@ -749,27 +749,27 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
+          <t>c1e0447b-a06c-44c8-abd0-3108b2f00b7a</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Broken link (connection error): https://www2.gov.bc.ca/gov/content/data/geographic-data-services/topographic-data/freshwater</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>f1f4ee29-1d0d-49f9-9a5b-64768f24a6ff</t>
+          <t>c1e0447b-a06c-44c8-abd0-3108b2f00b7a</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/file/d/1GWVbbZg0UM-0GLQA9urqg4uySDrLPr6D/view?usp=sharing returned status_code=500</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -779,70 +779,25 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>c7a168e8-f15e-446f-a49d-0b4a1f043ac2</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Broken link (202): https://fjedna.shinyapps.io/census-app1/</t>
+          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>c1e0447b-a06c-44c8-abd0-3108b2f00b7a</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
-        <is>
-          <t>No version</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="n">
-        <v>1</v>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>c1e0447b-a06c-44c8-abd0-3108b2f00b7a</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>No DOI defined</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="n">
-        <v>0</v>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="n">
-        <v>1</v>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
         <is>
           <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
         </is>

</xml_diff>

<commit_message>
Deployed f372394ba to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/issues_list.xlsx
+++ b/main/issues_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -434,12 +434,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
+          <t>646dd927-3248-4fc9-970c-abea15f7d304</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Hakai Institute' in DataCite not found in CKAN record</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -449,42 +449,42 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
+          <t>646dd927-3248-4fc9-970c-abea15f7d304</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Government of British Columbia' in DataCite not found in CKAN record</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
+          <t>bd461764-55b0-4c63-935a-5e9d1d5a6fed</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'Hakai Geospatial' in CKAN record not found in DataCite</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-itracksept2023 returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>b6621a3c-1700-4015-a359-56b6c7155835</t>
+          <t>da040f55-984d-490d-b917-a67856de4bac</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Metadata mismatch: author 'GeoBC Branch' in CKAN record not found in DataCite</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-seastars2024 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -494,27 +494,27 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>646dd927-3248-4fc9-970c-abea15f7d304</t>
+          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>646dd927-3248-4fc9-970c-abea15f7d304</t>
+          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -524,12 +524,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>bd461764-55b0-4c63-935a-5e9d1d5a6fed</t>
+          <t>c4932b55-1dd8-4f2f-89da-5822056ecc37</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-itracksept2023 returned status_code=404</t>
+          <t>Broken link (404): https://doi.org/10.21966/ekwk-r335</t>
         </is>
       </c>
     </row>
@@ -539,12 +539,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>da040f55-984d-490d-b917-a67856de4bac</t>
+          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-seastars2024 returned status_code=404</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -554,12 +554,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
+          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
+          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-qu5-mooring-data</t>
         </is>
       </c>
     </row>
@@ -569,12 +569,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>432b05ce-8904-4094-94bf-b97fb6636e41</t>
+          <t>33bb67af-4d61-4b15-93a9-f3ab2498430b</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Record DOI HTTPS link is failling: https://doi.org/10.21966/kp87-sf64 status_code=502</t>
+          <t>Broken link (404): http://www.env.gov.bc.ca/omfd/reports/Kelp2007-HakaiPass.pdf</t>
         </is>
       </c>
     </row>
@@ -584,12 +584,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
+          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -599,12 +599,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>c4932b55-1dd8-4f2f-89da-5822056ecc37</t>
+          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Broken link (404): https://doi.org/10.21966/ekwk-r335</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -614,27 +614,27 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>33bb67af-4d61-4b15-93a9-f3ab2498430b</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Broken link (404): http://www.env.gov.bc.ca/omfd/reports/Kelp2007-HakaiPass.pdf</t>
+          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
         </is>
       </c>
     </row>
@@ -644,27 +644,27 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-qu5-mooring-data</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -674,12 +674,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
+          <t>c7a168e8-f15e-446f-a49d-0b4a1f043ac2</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
+          <t>Broken link (202): https://fjedna.shinyapps.io/census-app1/</t>
         </is>
       </c>
     </row>
@@ -689,12 +689,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>c1e0447b-a06c-44c8-abd0-3108b2f00b7a</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
+          <t>No version</t>
         </is>
       </c>
     </row>
@@ -704,12 +704,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>c1e0447b-a06c-44c8-abd0-3108b2f00b7a</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -719,12 +719,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
         </is>
       </c>
     </row>
@@ -734,12 +734,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
         </is>
       </c>
     </row>
@@ -749,57 +749,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>c1e0447b-a06c-44c8-abd0-3108b2f00b7a</t>
+          <t>8882a149-fabd-4ecd-98d3-68a2a88aee38</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>No version</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="n">
-        <v>1</v>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>c1e0447b-a06c-44c8-abd0-3108b2f00b7a</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>No DOI defined</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="n">
-        <v>0</v>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="n">
-        <v>1</v>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+          <t>Invalid Resource URL: http://docs.turnerdesigns.com/t2/doc/manuals/998-7210.pdf returned status_code=timeout</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deployed 036594a43 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/issues_list.xlsx
+++ b/main/issues_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -460,7 +460,7 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -475,7 +475,7 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -490,7 +490,7 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -505,7 +505,7 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -520,7 +520,7 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -535,7 +535,7 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -550,7 +550,7 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -565,241 +565,226 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
+          <t>5042c858-d375-42f5-82e0-ee1e4da962b6</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
+          <t>Metadata mismatch: version CKAN='1.4' | DataCite='1.5'</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
+          <t>5042c858-d375-42f5-82e0-ee1e4da962b6</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-qu5-mooring-data</t>
+          <t>Metadata mismatch: publication year CKAN='2024' | DataCite='2026'</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
+          <t>5042c858-d375-42f5-82e0-ee1e4da962b6</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
+          <t>Metadata mismatch: related identifier 'https://doi.org/10.3389/fmars.2024.1458677' (IsPublishedIn) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
+          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-qu5-mooring-data</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
+          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Broken link (connection error): https://www2.gov.bc.ca/gov/content/data/geographic-data-services/topographic-data/freshwater</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>c7a168e8-f15e-446f-a49d-0b4a1f043ac2</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Broken link (202): https://fjedna.shinyapps.io/census-app1/</t>
+          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>c7a168e8-f15e-446f-a49d-0b4a1f043ac2</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+          <t>Broken link (202): https://fjedna.shinyapps.io/census-app1/</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>098c52a1-6dde-4e64-8b27-5a34e40870e6</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Broken link (502): https://doi.org/10.21966/pk18-z035</t>
+          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>c83b5cbf-cc8c-4676-823c-77e28c0ec9da</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=14Bgz48Ypo3Tt6W5sXHruSdvgC7HmrN5X returned status_code=500</t>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>d269f354-8527-4e94-bb32-9de4fe3fabdf</t>
+          <t>acd6c43f-6cbd-43c8-9bff-7d9ae6630295</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Contact missing ORCID: Sheridan, Kate</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="n">
-        <v>24</v>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>d269f354-8527-4e94-bb32-9de4fe3fabdf</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Contact missing ORCID: Sunday, Jennifer</t>
+          <t>Invalid Resource URL: https://catalogue.hakai.org/erddap/tabledap/HakaiWaterPropertiesInstrumentProfileProvisional.nc?work_area%2Ccruise%2Chakai_id%2Cvessel%2Coperators%2Ccomments%2Cdevice_model%2Cdevice_sn%2Cdevice_firmware%2Ccast_processing_stage%2Cstation%2Clatitude%2Clongitude%2Cprecise_latitude%2Cprecise_longitude%2Ctime%2Cbottom_date_time%2Cend_date_time%2Cmeasurement_date_time%2Cbottom_depth%2Ctarget_depth%2Cdrop_speed%2Cdirection_flag%2Cdescent_rate%2Cdepth%2Cdepth_UQL%2Cdepth_flag_description%2Cpressure%2Cpressure_UQL%2Cpressure_flag_description%2Cconductivity%2Cconductivity_UQL%2Cconductivity_flag_description%2Ctemperature%2Ctemperature_UQL%2Ctemperature_flag_description%2Csalinity%2Csalinity_UQL%2Csalinity_flag_description%2Cdissolved_oxygen_ml_l%2Cdissolved_oxygen_ml_l_UQL%2Cdissolved_oxygen_ml_l_flag_description%2Crinko_do_ml_l%2Crinko_do_ml_l_UQL%2Crinko_do_ml_l_flag_description%2Cflc%2Cflc_UQL%2Cflc_flag_description%2Cturbidity%2Cturbidity_UQL%2Cturbidity_flag_description%2Cpar%2Cpar_UQL%2Cpar_flag_description%2Cc_star_at%2Cc_star_at_UQL%2Cc_star_at_flag_description%2Cph%2Cph_UQL%2Ccph_flag_description%2Cbackscatter_beta%2Cbackscatter_beta_UQL%2Cbackscatter_beta_flag_description%2Ccdom_ppb%2Ccdom_ppb_UQL%2Ccdom_flag_description&amp;work_area=~%22QUADRA%7CJOHNSTONE%20STRAIT%22&amp;cruise=~%22JS%7CJS%20C%7CJS1%7CJS12%7CJSA1%7CJSA2%7CJSB%7CJSC%7CJSSOCKEYE%7COTHER%2CJSSOCKEYE%7CDI_C%2CDISOCKEYE%7CDI_W%2CDISOCKEYE%7CDISOCKEYE%22 returned status_code=502</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deployed ac8f2f727 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/issues_list.xlsx
+++ b/main/issues_list.xlsx
@@ -569,42 +569,42 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>5042c858-d375-42f5-82e0-ee1e4da962b6</t>
+          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Metadata mismatch: version CKAN='1.4' | DataCite='1.5'</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>5042c858-d375-42f5-82e0-ee1e4da962b6</t>
+          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Metadata mismatch: publication year CKAN='2024' | DataCite='2026'</t>
+          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-qu5-mooring-data</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>5042c858-d375-42f5-82e0-ee1e4da962b6</t>
+          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://doi.org/10.3389/fmars.2024.1458677' (IsPublishedIn) in DataCite not found in CKAN</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -614,12 +614,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
+          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -629,27 +629,27 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-qu5-mooring-data</t>
+          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
         </is>
       </c>
     </row>
@@ -659,18 +659,18 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -679,22 +679,22 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>c7a168e8-f15e-446f-a49d-0b4a1f043ac2</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Broken link (202): https://fjedna.shinyapps.io/census-app1/</t>
         </is>
       </c>
     </row>
@@ -704,7 +704,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -719,7 +719,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -734,42 +734,42 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>c7a168e8-f15e-446f-a49d-0b4a1f043ac2</t>
+          <t>186d3139-66a1-43f9-9ac7-c5607252146e</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Broken link (202): https://fjedna.shinyapps.io/census-app1/</t>
+          <t>Metadata mismatch: version CKAN='1.0' | DataCite='1.1'</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>186d3139-66a1-43f9-9ac7-c5607252146e</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
+          <t>Metadata mismatch: publication year CKAN='2025' | DataCite='2026'</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>186d3139-66a1-43f9-9ac7-c5607252146e</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+          <t>Metadata mismatch: creator 'Jon Bergshoeff' in DataCite not found in CKAN record</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deployed c43e75b71 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/issues_list.xlsx
+++ b/main/issues_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -634,7 +634,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
         </is>
       </c>
     </row>
@@ -649,7 +649,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
         </is>
       </c>
     </row>
@@ -709,7 +709,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
         </is>
       </c>
     </row>
@@ -724,67 +724,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="n">
-        <v>0</v>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>186d3139-66a1-43f9-9ac7-c5607252146e</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: version CKAN='1.0' | DataCite='1.1'</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="n">
-        <v>1</v>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>186d3139-66a1-43f9-9ac7-c5607252146e</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: publication year CKAN='2025' | DataCite='2026'</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="n">
-        <v>2</v>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>186d3139-66a1-43f9-9ac7-c5607252146e</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: creator 'Jon Bergshoeff' in DataCite not found in CKAN record</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="n">
-        <v>0</v>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>acd6c43f-6cbd-43c8-9bff-7d9ae6630295</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Invalid Resource URL: https://catalogue.hakai.org/erddap/tabledap/HakaiWaterPropertiesInstrumentProfileProvisional.nc?work_area%2Ccruise%2Chakai_id%2Cvessel%2Coperators%2Ccomments%2Cdevice_model%2Cdevice_sn%2Cdevice_firmware%2Ccast_processing_stage%2Cstation%2Clatitude%2Clongitude%2Cprecise_latitude%2Cprecise_longitude%2Ctime%2Cbottom_date_time%2Cend_date_time%2Cmeasurement_date_time%2Cbottom_depth%2Ctarget_depth%2Cdrop_speed%2Cdirection_flag%2Cdescent_rate%2Cdepth%2Cdepth_UQL%2Cdepth_flag_description%2Cpressure%2Cpressure_UQL%2Cpressure_flag_description%2Cconductivity%2Cconductivity_UQL%2Cconductivity_flag_description%2Ctemperature%2Ctemperature_UQL%2Ctemperature_flag_description%2Csalinity%2Csalinity_UQL%2Csalinity_flag_description%2Cdissolved_oxygen_ml_l%2Cdissolved_oxygen_ml_l_UQL%2Cdissolved_oxygen_ml_l_flag_description%2Crinko_do_ml_l%2Crinko_do_ml_l_UQL%2Crinko_do_ml_l_flag_description%2Cflc%2Cflc_UQL%2Cflc_flag_description%2Cturbidity%2Cturbidity_UQL%2Cturbidity_flag_description%2Cpar%2Cpar_UQL%2Cpar_flag_description%2Cc_star_at%2Cc_star_at_UQL%2Cc_star_at_flag_description%2Cph%2Cph_UQL%2Ccph_flag_description%2Cbackscatter_beta%2Cbackscatter_beta_UQL%2Cbackscatter_beta_flag_description%2Ccdom_ppb%2Ccdom_ppb_UQL%2Ccdom_flag_description&amp;work_area=~%22QUADRA%7CJOHNSTONE%20STRAIT%22&amp;cruise=~%22JS%7CJS%20C%7CJS1%7CJS12%7CJSA1%7CJSA2%7CJSB%7CJSC%7CJSSOCKEYE%7COTHER%2CJSSOCKEYE%7CDI_C%2CDISOCKEYE%7CDI_W%2CDISOCKEYE%7CDISOCKEYE%22 returned status_code=502</t>
+          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deployed e6f19fe3b to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/issues_list.xlsx
+++ b/main/issues_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -494,12 +494,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
+          <t>227eb965-1892-4bad-8ded-dd2e1d68fdf6</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
+          <t>Invalid Resource URL: https://www.ncbi.nlm.nih.gov/bioproject/PRJNA1269471 returned status_code=500</t>
         </is>
       </c>
     </row>
@@ -509,12 +509,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
+          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -524,12 +524,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>c4932b55-1dd8-4f2f-89da-5822056ecc37</t>
+          <t>44bdc298-1329-400a-bc02-4d35d251865d</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Broken link (404): https://doi.org/10.21966/ekwk-r335</t>
+          <t>Invalid Resource URL: http://www.ncbi.nlm.nih.gov/bioproject/1049344 returned status_code=500</t>
         </is>
       </c>
     </row>
@@ -539,27 +539,27 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>1e13d2ee-580f-4785-838b-908a449781a3</t>
+          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>1e13d2ee-580f-4785-838b-908a449781a3</t>
+          <t>2de051d0-4deb-4d0a-ad22-96fd660e6276</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/GEM-Kit10-repository/tree/main returned status_code=404</t>
+          <t>Invalid Resource URL: https://www.ncbi.nlm.nih.gov/bioproject/PRJNA937254/ returned status_code=500</t>
         </is>
       </c>
     </row>
@@ -569,12 +569,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
+          <t>c4932b55-1dd8-4f2f-89da-5822056ecc37</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
+          <t>Broken link (404): https://doi.org/10.21966/ekwk-r335</t>
         </is>
       </c>
     </row>
@@ -584,12 +584,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
+          <t>e14d0456-297e-4636-8e7c-c615791b165e</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-qu5-mooring-data</t>
+          <t>Invalid Resource URL: https://www.ncbi.nlm.nih.gov/bioproject/PRJNA1456220 returned status_code=500</t>
         </is>
       </c>
     </row>
@@ -599,27 +599,27 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
+          <t>1e13d2ee-580f-4785-838b-908a449781a3</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
+          <t>1e13d2ee-580f-4785-838b-908a449781a3</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/GEM-Kit10-repository/tree/main returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -629,27 +629,27 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
+          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-qu5-mooring-data</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -659,27 +659,27 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>5c2aac2c-0dd8-49d8-87b2-5c52b3d42946</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Invalid Resource URL: https://www.ncbi.nlm.nih.gov/bioproject/PRJNA865652/ returned status_code=500</t>
         </is>
       </c>
     </row>
@@ -689,12 +689,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>c7a168e8-f15e-446f-a49d-0b4a1f043ac2</t>
+          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Broken link (202): https://fjedna.shinyapps.io/census-app1/</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -704,12 +704,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
         </is>
       </c>
     </row>
@@ -719,12 +719,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
         </is>
       </c>
     </row>
@@ -734,12 +734,177 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>acd6c43f-6cbd-43c8-9bff-7d9ae6630295</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://catalogue.hakai.org/erddap/tabledap/HakaiWaterPropertiesInstrumentProfileProvisional.nc?work_area%2Ccruise%2Chakai_id%2Cvessel%2Coperators%2Ccomments%2Cdevice_model%2Cdevice_sn%2Cdevice_firmware%2Ccast_processing_stage%2Cstation%2Clatitude%2Clongitude%2Cprecise_latitude%2Cprecise_longitude%2Ctime%2Cbottom_date_time%2Cend_date_time%2Cmeasurement_date_time%2Cbottom_depth%2Ctarget_depth%2Cdrop_speed%2Cdirection_flag%2Cdescent_rate%2Cdepth%2Cdepth_UQL%2Cdepth_flag_description%2Cpressure%2Cpressure_UQL%2Cpressure_flag_description%2Cconductivity%2Cconductivity_UQL%2Cconductivity_flag_description%2Ctemperature%2Ctemperature_UQL%2Ctemperature_flag_description%2Csalinity%2Csalinity_UQL%2Csalinity_flag_description%2Cdissolved_oxygen_ml_l%2Cdissolved_oxygen_ml_l_UQL%2Cdissolved_oxygen_ml_l_flag_description%2Crinko_do_ml_l%2Crinko_do_ml_l_UQL%2Crinko_do_ml_l_flag_description%2Cflc%2Cflc_UQL%2Cflc_flag_description%2Cturbidity%2Cturbidity_UQL%2Cturbidity_flag_description%2Cpar%2Cpar_UQL%2Cpar_flag_description%2Cc_star_at%2Cc_star_at_UQL%2Cc_star_at_flag_description%2Cph%2Cph_UQL%2Ccph_flag_description%2Cbackscatter_beta%2Cbackscatter_beta_UQL%2Cbackscatter_beta_flag_description%2Ccdom_ppb%2Ccdom_ppb_UQL%2Ccdom_flag_description&amp;work_area=~%22QUADRA%7CJOHNSTONE%20STRAIT%22&amp;cruise=~%22JS%7CJS%20C%7CJS1%7CJS12%7CJSA1%7CJSA2%7CJSB%7CJSC%7CJSSOCKEYE%7COTHER%2CJSSOCKEYE%7CDI_C%2CDISOCKEYE%7CDI_W%2CDISOCKEYE%7CDISOCKEYE%22 returned status_code=502</t>
+          <t>No DOI defined</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>1</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>No funder</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>0</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Broken link (connection error): https://www2.gov.bc.ca/gov/content/data/geographic-data-services/topographic-data/freshwater</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>0</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>c5e60545-c6f2-4945-af0a-21812ba5f0d9</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Invalid Resource URL: https://www.ncbi.nlm.nih.gov/bioproject/1269473 returned status_code=500</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>0</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>1</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>0</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>c7a168e8-f15e-446f-a49d-0b4a1f043ac2</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Record DOI HTTPS link is failling: https://doi.org/10.21966/n141-m959 status_code=502</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>1</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>c7a168e8-f15e-446f-a49d-0b4a1f043ac2</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Invalid Resource URL: https://www.ncbi.nlm.nih.gov/bioproject/?term=1289220 returned status_code=500</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>2</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>c7a168e8-f15e-446f-a49d-0b4a1f043ac2</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Broken link (202): https://fjedna.shinyapps.io/census-app1/</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>0</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>6be4c552-469a-4558-b63d-7a2c52566fe2</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Invalid Resource URL: https://www.ncbi.nlm.nih.gov/bioproject/?term=PRJNA1195080 returned status_code=500</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>1</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>6be4c552-469a-4558-b63d-7a2c52566fe2</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Invalid Resource URL: https://www.ncbi.nlm.nih.gov/bioproject/1232168/ returned status_code=500</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>0</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>d269f354-8527-4e94-bb32-9de4fe3fabdf</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Invalid Resource URL: https://www.ncbi.nlm.nih.gov/bioproject/PRJNA1037528/ returned status_code=500</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deployed 5d47a73da to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/issues_list.xlsx
+++ b/main/issues_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C33"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -494,12 +494,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>227eb965-1892-4bad-8ded-dd2e1d68fdf6</t>
+          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://www.ncbi.nlm.nih.gov/bioproject/PRJNA1269471 returned status_code=500</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -509,12 +509,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
+          <t>227eb965-1892-4bad-8ded-dd2e1d68fdf6</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
+          <t>Invalid Resource URL: https://www.ncbi.nlm.nih.gov/bioproject/PRJNA1269471 returned status_code=500</t>
         </is>
       </c>
     </row>
@@ -524,12 +524,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>44bdc298-1329-400a-bc02-4d35d251865d</t>
+          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: http://www.ncbi.nlm.nih.gov/bioproject/1049344 returned status_code=500</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -539,12 +539,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
+          <t>44bdc298-1329-400a-bc02-4d35d251865d</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
+          <t>Invalid Resource URL: http://www.ncbi.nlm.nih.gov/bioproject/1049344 returned status_code=500</t>
         </is>
       </c>
     </row>
@@ -554,12 +554,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2de051d0-4deb-4d0a-ad22-96fd660e6276</t>
+          <t>c4932b55-1dd8-4f2f-89da-5822056ecc37</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://www.ncbi.nlm.nih.gov/bioproject/PRJNA937254/ returned status_code=500</t>
+          <t>Broken link (404): https://doi.org/10.21966/ekwk-r335</t>
         </is>
       </c>
     </row>
@@ -569,12 +569,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>c4932b55-1dd8-4f2f-89da-5822056ecc37</t>
+          <t>e14d0456-297e-4636-8e7c-c615791b165e</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Broken link (404): https://doi.org/10.21966/ekwk-r335</t>
+          <t>Invalid Resource URL: https://www.ncbi.nlm.nih.gov/bioproject/PRJNA1456220 returned status_code=500</t>
         </is>
       </c>
     </row>
@@ -584,18 +584,18 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>e14d0456-297e-4636-8e7c-c615791b165e</t>
+          <t>1e13d2ee-580f-4785-838b-908a449781a3</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://www.ncbi.nlm.nih.gov/bioproject/PRJNA1456220 returned status_code=500</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -604,22 +604,22 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/GEM-Kit10-repository/tree/main returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>1e13d2ee-580f-4785-838b-908a449781a3</t>
+          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/GEM-Kit10-repository/tree/main returned status_code=404</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -629,12 +629,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
+          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-qu5-mooring-data</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -644,12 +644,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
+          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -659,12 +659,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
+          <t>5c2aac2c-0dd8-49d8-87b2-5c52b3d42946</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
+          <t>Invalid Resource URL: https://www.ncbi.nlm.nih.gov/bioproject/PRJNA865652/ returned status_code=500</t>
         </is>
       </c>
     </row>
@@ -674,27 +674,27 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>5c2aac2c-0dd8-49d8-87b2-5c52b3d42946</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://www.ncbi.nlm.nih.gov/bioproject/PRJNA865652/ returned status_code=500</t>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
+          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
         </is>
       </c>
     </row>
@@ -704,12 +704,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -719,12 +719,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -734,42 +734,42 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>c5e60545-c6f2-4945-af0a-21812ba5f0d9</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Invalid Resource URL: https://www.ncbi.nlm.nih.gov/bioproject/1269473 returned status_code=500</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Broken link (connection error): https://www2.gov.bc.ca/gov/content/data/geographic-data-services/topographic-data/freshwater</t>
+          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
         </is>
       </c>
     </row>
@@ -779,12 +779,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>c5e60545-c6f2-4945-af0a-21812ba5f0d9</t>
+          <t>c7a168e8-f15e-446f-a49d-0b4a1f043ac2</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://www.ncbi.nlm.nih.gov/bioproject/1269473 returned status_code=500</t>
+          <t>Broken link (202): https://fjedna.shinyapps.io/census-app1/</t>
         </is>
       </c>
     </row>
@@ -794,115 +794,25 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>6be4c552-469a-4558-b63d-7a2c52566fe2</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+          <t>Invalid Resource URL: https://www.ncbi.nlm.nih.gov/bioproject/1232168/ returned status_code=500</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>d269f354-8527-4e94-bb32-9de4fe3fabdf</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
-        <is>
-          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="n">
-        <v>0</v>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>c7a168e8-f15e-446f-a49d-0b4a1f043ac2</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>Record DOI HTTPS link is failling: https://doi.org/10.21966/n141-m959 status_code=502</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="n">
-        <v>1</v>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>c7a168e8-f15e-446f-a49d-0b4a1f043ac2</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Invalid Resource URL: https://www.ncbi.nlm.nih.gov/bioproject/?term=1289220 returned status_code=500</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="n">
-        <v>2</v>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>c7a168e8-f15e-446f-a49d-0b4a1f043ac2</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Broken link (202): https://fjedna.shinyapps.io/census-app1/</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="n">
-        <v>0</v>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>6be4c552-469a-4558-b63d-7a2c52566fe2</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>Invalid Resource URL: https://www.ncbi.nlm.nih.gov/bioproject/?term=PRJNA1195080 returned status_code=500</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="n">
-        <v>1</v>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>6be4c552-469a-4558-b63d-7a2c52566fe2</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>Invalid Resource URL: https://www.ncbi.nlm.nih.gov/bioproject/1232168/ returned status_code=500</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="n">
-        <v>0</v>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>d269f354-8527-4e94-bb32-9de4fe3fabdf</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
         <is>
           <t>Invalid Resource URL: https://www.ncbi.nlm.nih.gov/bioproject/PRJNA1037528/ returned status_code=500</t>
         </is>

</xml_diff>

<commit_message>
Deployed a1a36a0c9 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/issues_list.xlsx
+++ b/main/issues_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -509,12 +509,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>227eb965-1892-4bad-8ded-dd2e1d68fdf6</t>
+          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://www.ncbi.nlm.nih.gov/bioproject/PRJNA1269471 returned status_code=500</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -524,12 +524,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
+          <t>78efda1b-9688-4bcf-b16e-7167c17c0bcb</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
+          <t>Invalid Resource URL: https://drive.google.com/file/d/1darjhrdMVVZESNy0D_8aRbos95RkUfjR/view?usp=drive_link returned status_code=500</t>
         </is>
       </c>
     </row>
@@ -539,12 +539,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>44bdc298-1329-400a-bc02-4d35d251865d</t>
+          <t>c4932b55-1dd8-4f2f-89da-5822056ecc37</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: http://www.ncbi.nlm.nih.gov/bioproject/1049344 returned status_code=500</t>
+          <t>Broken link (404): https://doi.org/10.21966/ekwk-r335</t>
         </is>
       </c>
     </row>
@@ -554,27 +554,27 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>c4932b55-1dd8-4f2f-89da-5822056ecc37</t>
+          <t>1e13d2ee-580f-4785-838b-908a449781a3</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Broken link (404): https://doi.org/10.21966/ekwk-r335</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>e14d0456-297e-4636-8e7c-c615791b165e</t>
+          <t>1e13d2ee-580f-4785-838b-908a449781a3</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://www.ncbi.nlm.nih.gov/bioproject/PRJNA1456220 returned status_code=500</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/GEM-Kit10-repository/tree/main returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -584,27 +584,27 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>1e13d2ee-580f-4785-838b-908a449781a3</t>
+          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>1e13d2ee-580f-4785-838b-908a449781a3</t>
+          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/GEM-Kit10-repository/tree/main returned status_code=404</t>
+          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-qu5-mooring-data</t>
         </is>
       </c>
     </row>
@@ -614,12 +614,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
+          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -629,12 +629,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
+          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -644,27 +644,27 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>5c2aac2c-0dd8-49d8-87b2-5c52b3d42946</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://www.ncbi.nlm.nih.gov/bioproject/PRJNA865652/ returned status_code=500</t>
+          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
         </is>
       </c>
     </row>
@@ -674,12 +674,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
@@ -689,12 +689,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -704,42 +704,42 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>c7a168e8-f15e-446f-a49d-0b4a1f043ac2</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Broken link (202): https://fjedna.shinyapps.io/census-app1/</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>c5e60545-c6f2-4945-af0a-21812ba5f0d9</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://www.ncbi.nlm.nih.gov/bioproject/1269473 returned status_code=500</t>
+          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
         </is>
       </c>
     </row>
@@ -749,72 +749,27 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>826d8228-baab-4191-82de-44701cd93806</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+          <t>Invalid Resource URL: https://drive.google.com/file/d/1rJ4YH9pCDXLh60BI0vVaRYDyB3jrdcnp/view?usp=sharing returned status_code=500</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>acd6c43f-6cbd-43c8-9bff-7d9ae6630295</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="n">
-        <v>0</v>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>c7a168e8-f15e-446f-a49d-0b4a1f043ac2</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Broken link (202): https://fjedna.shinyapps.io/census-app1/</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="n">
-        <v>0</v>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>6be4c552-469a-4558-b63d-7a2c52566fe2</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Invalid Resource URL: https://www.ncbi.nlm.nih.gov/bioproject/1232168/ returned status_code=500</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="n">
-        <v>0</v>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>d269f354-8527-4e94-bb32-9de4fe3fabdf</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Invalid Resource URL: https://www.ncbi.nlm.nih.gov/bioproject/PRJNA1037528/ returned status_code=500</t>
+          <t>Invalid Resource URL: https://catalogue.hakai.org/erddap/tabledap/HakaiWaterPropertiesInstrumentProfileProvisional.nc?work_area%2Ccruise%2Chakai_id%2Cvessel%2Coperators%2Ccomments%2Cdevice_model%2Cdevice_sn%2Cdevice_firmware%2Ccast_processing_stage%2Cstation%2Clatitude%2Clongitude%2Cprecise_latitude%2Cprecise_longitude%2Ctime%2Cbottom_date_time%2Cend_date_time%2Cmeasurement_date_time%2Cbottom_depth%2Ctarget_depth%2Cdrop_speed%2Cdirection_flag%2Cdescent_rate%2Cdepth%2Cdepth_UQL%2Cdepth_flag_description%2Cpressure%2Cpressure_UQL%2Cpressure_flag_description%2Cconductivity%2Cconductivity_UQL%2Cconductivity_flag_description%2Ctemperature%2Ctemperature_UQL%2Ctemperature_flag_description%2Csalinity%2Csalinity_UQL%2Csalinity_flag_description%2Cdissolved_oxygen_ml_l%2Cdissolved_oxygen_ml_l_UQL%2Cdissolved_oxygen_ml_l_flag_description%2Crinko_do_ml_l%2Crinko_do_ml_l_UQL%2Crinko_do_ml_l_flag_description%2Cflc%2Cflc_UQL%2Cflc_flag_description%2Cturbidity%2Cturbidity_UQL%2Cturbidity_flag_description%2Cpar%2Cpar_UQL%2Cpar_flag_description%2Cc_star_at%2Cc_star_at_UQL%2Cc_star_at_flag_description%2Cph%2Cph_UQL%2Ccph_flag_description%2Cbackscatter_beta%2Cbackscatter_beta_UQL%2Cbackscatter_beta_flag_description%2Ccdom_ppb%2Ccdom_ppb_UQL%2Ccdom_flag_description&amp;work_area=~%22QUADRA%7CJOHNSTONE%20STRAIT%22&amp;cruise=~%22JS%7CJS%20C%7CJS1%7CJS12%7CJSA1%7CJSA2%7CJSB%7CJSC%7CJSSOCKEYE%7COTHER%2CJSSOCKEYE%7CDI_C%2CDISOCKEYE%7CDI_W%2CDISOCKEYE%7CDISOCKEYE%22 returned status_code=502</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deployed cbb638ef0 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/issues_list.xlsx
+++ b/main/issues_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:C29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -539,12 +539,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>e14d0456-297e-4636-8e7c-c615791b165e</t>
+          <t>4fe1609e-ce10-457e-bcf6-86918a5836ad</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://www.ncbi.nlm.nih.gov/bioproject/PRJNA1456220 returned status_code=404</t>
+          <t>Invalid Resource URL: https://www.ncbi.nlm.nih.gov/bioproject/PRJNA1538264 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -554,12 +554,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>4fe1609e-ce10-457e-bcf6-86918a5836ad</t>
+          <t>e14d0456-297e-4636-8e7c-c615791b165e</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://www.ncbi.nlm.nih.gov/bioproject/PRJNA1538264 returned status_code=404</t>
+          <t>Invalid Resource URL: https://www.ncbi.nlm.nih.gov/bioproject/PRJNA1456220 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -614,12 +614,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>5c2aac2c-0dd8-49d8-87b2-5c52b3d42946</t>
+          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://www.ncbi.nlm.nih.gov/bioproject/PRJNA865652/ returned status_code=404</t>
+          <t>Broken link (500): https://drive.google.com/file/d/1MT2v_uv78afJP5z_LHi1GU52BqwkO4ms/view?usp=drive_link</t>
         </is>
       </c>
     </row>
@@ -629,18 +629,18 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>1e13d2ee-580f-4785-838b-908a449781a3</t>
+          <t>5c2aac2c-0dd8-49d8-87b2-5c52b3d42946</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Invalid Resource URL: https://www.ncbi.nlm.nih.gov/bioproject/PRJNA865652/ returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -649,22 +649,22 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/GEM-Kit10-repository/tree/main returned status_code=404</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
+          <t>1e13d2ee-580f-4785-838b-908a449781a3</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/GEM-Kit10-repository/tree/main returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -674,12 +674,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
+          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-qu5-mooring-data</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -689,12 +689,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
+          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
+          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-qu5-mooring-data</t>
         </is>
       </c>
     </row>
@@ -704,12 +704,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
+          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -719,18 +719,18 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -745,22 +745,22 @@
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -769,22 +769,22 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>c7a168e8-f15e-446f-a49d-0b4a1f043ac2</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Broken link (202): https://fjedna.shinyapps.io/census-app1/</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -794,18 +794,18 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>c7a168e8-f15e-446f-a49d-0b4a1f043ac2</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
+          <t>Broken link (202): https://fjedna.shinyapps.io/census-app1/</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -820,14 +820,29 @@
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>0</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
           <t>d269f354-8527-4e94-bb32-9de4fe3fabdf</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>Invalid Resource URL: https://www.ncbi.nlm.nih.gov/bioproject/PRJNA1037528/ returned status_code=404</t>
         </is>

</xml_diff>

<commit_message>
Deployed a9cef2efa to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/issues_list.xlsx
+++ b/main/issues_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -434,12 +434,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>227eb965-1892-4bad-8ded-dd2e1d68fdf6</t>
+          <t>bd461764-55b0-4c63-935a-5e9d1d5a6fed</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://www.ncbi.nlm.nih.gov/bioproject/PRJNA1269471 returned status_code=404</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-itracksept2023 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -449,27 +449,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>646dd927-3248-4fc9-970c-abea15f7d304</t>
+          <t>da040f55-984d-490d-b917-a67856de4bac</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-seastars2024 returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>646dd927-3248-4fc9-970c-abea15f7d304</t>
+          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -479,12 +479,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>bd461764-55b0-4c63-935a-5e9d1d5a6fed</t>
+          <t>4a949e26-fe94-4f63-a3c6-a62e19301102</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-itracksept2023 returned status_code=404</t>
+          <t>Broken link (502): https://obis.org/dataset/80afee46-3e18-4669-ad1b-00f71b0544f5</t>
         </is>
       </c>
     </row>
@@ -494,12 +494,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2de051d0-4deb-4d0a-ad22-96fd660e6276</t>
+          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://www.ncbi.nlm.nih.gov/bioproject/PRJNA937254/ returned status_code=404</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -509,12 +509,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>30560220-bc44-4020-b424-0abf617d1c00</t>
+          <t>96b5a7f2-5f23-413a-b060-d268bcff83ba</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Broken link (410): https://coastalmarginsnetwork.org/</t>
+          <t>Broken link (connection error): https://doi.org/10.25921/kmam-ct93</t>
         </is>
       </c>
     </row>
@@ -524,12 +524,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>da040f55-984d-490d-b917-a67856de4bac</t>
+          <t>c4932b55-1dd8-4f2f-89da-5822056ecc37</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-seastars2024 returned status_code=404</t>
+          <t>Broken link (404): https://doi.org/10.21966/ekwk-r335</t>
         </is>
       </c>
     </row>
@@ -539,12 +539,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>4fe1609e-ce10-457e-bcf6-86918a5836ad</t>
+          <t>2ec7aa05-6a81-4836-bf79-0893cef2db95</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://www.ncbi.nlm.nih.gov/bioproject/PRJNA1538264 returned status_code=404</t>
+          <t>Broken link (502): https://dspace.library.uvic.ca/handle/1828/9312</t>
         </is>
       </c>
     </row>
@@ -554,27 +554,27 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>e14d0456-297e-4636-8e7c-c615791b165e</t>
+          <t>1e13d2ee-580f-4785-838b-908a449781a3</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://www.ncbi.nlm.nih.gov/bioproject/PRJNA1456220 returned status_code=404</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
+          <t>1e13d2ee-580f-4785-838b-908a449781a3</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/GEM-Kit10-repository/tree/main returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -584,12 +584,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
+          <t>d64fd03b-46d4-4662-a123-c11bc42199b6</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
+          <t>Invalid Resource URL: https://drive.google.com/file/d/1NdD_GW7ImI5Z3_y92TXp03ZcX2PhrQxQ/view?usp=sharing returned status_code=500</t>
         </is>
       </c>
     </row>
@@ -599,12 +599,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>c4932b55-1dd8-4f2f-89da-5822056ecc37</t>
+          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Broken link (404): https://doi.org/10.21966/ekwk-r335</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -614,12 +614,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
+          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Broken link (500): https://drive.google.com/file/d/1MT2v_uv78afJP5z_LHi1GU52BqwkO4ms/view?usp=drive_link</t>
+          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-qu5-mooring-data</t>
         </is>
       </c>
     </row>
@@ -629,12 +629,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>5c2aac2c-0dd8-49d8-87b2-5c52b3d42946</t>
+          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://www.ncbi.nlm.nih.gov/bioproject/PRJNA865652/ returned status_code=404</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -644,42 +644,42 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>1e13d2ee-580f-4785-838b-908a449781a3</t>
+          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>1e13d2ee-580f-4785-838b-908a449781a3</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/GEM-Kit10-repository/tree/main returned status_code=404</t>
+          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
         </is>
       </c>
     </row>
@@ -689,27 +689,27 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-qu5-mooring-data</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -719,12 +719,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
+          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
+          <t>Broken link (connection error): https://www2.gov.bc.ca/gov/content/data/geographic-data-services/topographic-data/freshwater</t>
         </is>
       </c>
     </row>
@@ -734,22 +734,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>c7a168e8-f15e-446f-a49d-0b4a1f043ac2</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+          <t>Broken link (202): https://fjedna.shinyapps.io/census-app1/</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -760,91 +760,31 @@
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>8882a149-fabd-4ecd-98d3-68a2a88aee38</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>No funder</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="n">
-        <v>0</v>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>c7a168e8-f15e-446f-a49d-0b4a1f043ac2</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Broken link (202): https://fjedna.shinyapps.io/census-app1/</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="n">
-        <v>0</v>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="n">
-        <v>1</v>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="n">
-        <v>0</v>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>d269f354-8527-4e94-bb32-9de4fe3fabdf</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Invalid Resource URL: https://www.ncbi.nlm.nih.gov/bioproject/PRJNA1037528/ returned status_code=404</t>
+          <t>Invalid Resource URL: http://docs.turnerdesigns.com/t2/doc/manuals/998-7210.pdf returned status_code=timeout</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deployed 2f251c896 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/issues_list.xlsx
+++ b/main/issues_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -449,12 +449,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>da040f55-984d-490d-b917-a67856de4bac</t>
+          <t>30560220-bc44-4020-b424-0abf617d1c00</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-seastars2024 returned status_code=404</t>
+          <t>Broken link (410): https://coastalmarginsnetwork.org/</t>
         </is>
       </c>
     </row>
@@ -464,12 +464,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
+          <t>da040f55-984d-490d-b917-a67856de4bac</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-seastars2024 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -479,12 +479,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
+          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -494,12 +494,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>c4932b55-1dd8-4f2f-89da-5822056ecc37</t>
+          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Broken link (404): https://doi.org/10.21966/ekwk-r335</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -509,18 +509,18 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>1e13d2ee-580f-4785-838b-908a449781a3</t>
+          <t>c4932b55-1dd8-4f2f-89da-5822056ecc37</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Broken link (404): https://doi.org/10.21966/ekwk-r335</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -529,22 +529,22 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/GEM-Kit10-repository/tree/main returned status_code=404</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
+          <t>1e13d2ee-580f-4785-838b-908a449781a3</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/GEM-Kit10-repository/tree/main returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -554,12 +554,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
+          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-qu5-mooring-data</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -569,12 +569,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
+          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
+          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-qu5-mooring-data</t>
         </is>
       </c>
     </row>
@@ -584,12 +584,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
+          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -599,33 +599,33 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -640,31 +640,31 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
+          <t>No DOI defined</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>c7a168e8-f15e-446f-a49d-0b4a1f043ac2</t>
+          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Broken link (202): https://fjedna.shinyapps.io/census-app1/</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -674,18 +674,18 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>c7a168e8-f15e-446f-a49d-0b4a1f043ac2</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+          <t>Broken link (202): https://fjedna.shinyapps.io/census-app1/</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -700,14 +700,29 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>0</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
           <t>acd6c43f-6cbd-43c8-9bff-7d9ae6630295</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>Invalid Resource URL: https://catalogue.hakai.org/erddap/tabledap/HakaiWaterPropertiesInstrumentProfileProvisional.nc?work_area%2Ccruise%2Chakai_id%2Cvessel%2Coperators%2Ccomments%2Cdevice_model%2Cdevice_sn%2Cdevice_firmware%2Ccast_processing_stage%2Cstation%2Clatitude%2Clongitude%2Cprecise_latitude%2Cprecise_longitude%2Ctime%2Cbottom_date_time%2Cend_date_time%2Cmeasurement_date_time%2Cbottom_depth%2Ctarget_depth%2Cdrop_speed%2Cdirection_flag%2Cdescent_rate%2Cdepth%2Cdepth_UQL%2Cdepth_flag_description%2Cpressure%2Cpressure_UQL%2Cpressure_flag_description%2Cconductivity%2Cconductivity_UQL%2Cconductivity_flag_description%2Ctemperature%2Ctemperature_UQL%2Ctemperature_flag_description%2Csalinity%2Csalinity_UQL%2Csalinity_flag_description%2Cdissolved_oxygen_ml_l%2Cdissolved_oxygen_ml_l_UQL%2Cdissolved_oxygen_ml_l_flag_description%2Crinko_do_ml_l%2Crinko_do_ml_l_UQL%2Crinko_do_ml_l_flag_description%2Cflc%2Cflc_UQL%2Cflc_flag_description%2Cturbidity%2Cturbidity_UQL%2Cturbidity_flag_description%2Cpar%2Cpar_UQL%2Cpar_flag_description%2Cc_star_at%2Cc_star_at_UQL%2Cc_star_at_flag_description%2Cph%2Cph_UQL%2Ccph_flag_description%2Cbackscatter_beta%2Cbackscatter_beta_UQL%2Cbackscatter_beta_flag_description%2Ccdom_ppb%2Ccdom_ppb_UQL%2Ccdom_flag_description&amp;work_area=~%22QUADRA%7CJOHNSTONE%20STRAIT%22&amp;cruise=~%22JS%7CJS%20C%7CJS1%7CJS12%7CJSA1%7CJSA2%7CJSB%7CJSC%7CJSSOCKEYE%7COTHER%2CJSSOCKEYE%7CDI_C%2CDISOCKEYE%7CDI_W%2CDISOCKEYE%7CDISOCKEYE%22 returned status_code=502</t>
         </is>

</xml_diff>

<commit_message>
Deployed 0ee595148 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/issues_list.xlsx
+++ b/main/issues_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -449,12 +449,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>30560220-bc44-4020-b424-0abf617d1c00</t>
+          <t>da040f55-984d-490d-b917-a67856de4bac</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Broken link (410): https://coastalmarginsnetwork.org/</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-seastars2024 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -464,12 +464,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>da040f55-984d-490d-b917-a67856de4bac</t>
+          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-seastars2024 returned status_code=404</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -479,12 +479,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
+          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -494,12 +494,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
+          <t>c4932b55-1dd8-4f2f-89da-5822056ecc37</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
+          <t>Broken link (404): https://doi.org/10.21966/ekwk-r335</t>
         </is>
       </c>
     </row>
@@ -509,12 +509,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>c4932b55-1dd8-4f2f-89da-5822056ecc37</t>
+          <t>2ec7aa05-6a81-4836-bf79-0893cef2db95</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Broken link (404): https://doi.org/10.21966/ekwk-r335</t>
+          <t>Broken link (502): https://dspace.library.uvic.ca/handle/1828/9312</t>
         </is>
       </c>
     </row>
@@ -554,12 +554,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
+          <t>0cef18ab-cea6-4522-baba-1bcd73a30646</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
+          <t>Broken link (500): https://drive.google.com/file/d/10DXaHVFkhdYlkpgrMBW7Ie4wXWmScNZb/view?usp=drive_link</t>
         </is>
       </c>
     </row>
@@ -584,12 +584,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
+          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -599,12 +599,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
+          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -614,18 +614,18 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -634,37 +634,37 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>No DOI defined</t>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>49967494-a7b6-4128-b336-671971d1e2c6</t>
+          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Broken link (connection error): https://www2.gov.bc.ca/gov/content/data/geographic-data-services/topographic-data/freshwater</t>
         </is>
       </c>
     </row>
@@ -725,6 +725,21 @@
       <c r="C21" t="inlineStr">
         <is>
           <t>Invalid Resource URL: https://catalogue.hakai.org/erddap/tabledap/HakaiWaterPropertiesInstrumentProfileProvisional.nc?work_area%2Ccruise%2Chakai_id%2Cvessel%2Coperators%2Ccomments%2Cdevice_model%2Cdevice_sn%2Cdevice_firmware%2Ccast_processing_stage%2Cstation%2Clatitude%2Clongitude%2Cprecise_latitude%2Cprecise_longitude%2Ctime%2Cbottom_date_time%2Cend_date_time%2Cmeasurement_date_time%2Cbottom_depth%2Ctarget_depth%2Cdrop_speed%2Cdirection_flag%2Cdescent_rate%2Cdepth%2Cdepth_UQL%2Cdepth_flag_description%2Cpressure%2Cpressure_UQL%2Cpressure_flag_description%2Cconductivity%2Cconductivity_UQL%2Cconductivity_flag_description%2Ctemperature%2Ctemperature_UQL%2Ctemperature_flag_description%2Csalinity%2Csalinity_UQL%2Csalinity_flag_description%2Cdissolved_oxygen_ml_l%2Cdissolved_oxygen_ml_l_UQL%2Cdissolved_oxygen_ml_l_flag_description%2Crinko_do_ml_l%2Crinko_do_ml_l_UQL%2Crinko_do_ml_l_flag_description%2Cflc%2Cflc_UQL%2Cflc_flag_description%2Cturbidity%2Cturbidity_UQL%2Cturbidity_flag_description%2Cpar%2Cpar_UQL%2Cpar_flag_description%2Cc_star_at%2Cc_star_at_UQL%2Cc_star_at_flag_description%2Cph%2Cph_UQL%2Ccph_flag_description%2Cbackscatter_beta%2Cbackscatter_beta_UQL%2Cbackscatter_beta_flag_description%2Ccdom_ppb%2Ccdom_ppb_UQL%2Ccdom_flag_description&amp;work_area=~%22QUADRA%7CJOHNSTONE%20STRAIT%22&amp;cruise=~%22JS%7CJS%20C%7CJS1%7CJS12%7CJSA1%7CJSA2%7CJSB%7CJSC%7CJSSOCKEYE%7COTHER%2CJSSOCKEYE%7CDI_C%2CDISOCKEYE%7CDI_W%2CDISOCKEYE%7CDISOCKEYE%22 returned status_code=502</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>0</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>b01f58f7-1518-4829-aff6-ac4a8f2c0616</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Broken link (500): https://drive.google.com/file/d/1AvIuDRR06KE-z70reZmNMMbkYOU1Hzgo/view</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deployed 5045f061c to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/issues_list.xlsx
+++ b/main/issues_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -494,12 +494,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>876027b6-cf37-4d49-8c3d-22d40b5f5b0b</t>
+          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Record DOI HTTPS link is failling: https://doi.org/10.21966/1.715740 status_code=502</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -509,12 +509,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
+          <t>c4932b55-1dd8-4f2f-89da-5822056ecc37</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
+          <t>Broken link (404): https://doi.org/10.21966/ekwk-r335</t>
         </is>
       </c>
     </row>
@@ -524,18 +524,18 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>c4932b55-1dd8-4f2f-89da-5822056ecc37</t>
+          <t>1e13d2ee-580f-4785-838b-908a449781a3</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Broken link (404): https://doi.org/10.21966/ekwk-r335</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -544,22 +544,22 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/GEM-Kit10-repository/tree/main returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>1e13d2ee-580f-4785-838b-908a449781a3</t>
+          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/GEM-Kit10-repository/tree/main returned status_code=404</t>
+          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-qu5-mooring-data</t>
         </is>
       </c>
     </row>
@@ -569,12 +569,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
+          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -584,12 +584,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
+          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-qu5-mooring-data</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -599,27 +599,27 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
+          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
         </is>
       </c>
     </row>
@@ -629,27 +629,27 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+          <t>Broken link (connection error): https://www2.gov.bc.ca/gov/content/data/geographic-data-services/topographic-data/freshwater</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>c7a168e8-f15e-446f-a49d-0b4a1f043ac2</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
+          <t>Broken link (202): https://fjedna.shinyapps.io/census-app1/</t>
         </is>
       </c>
     </row>
@@ -659,18 +659,18 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>c7a168e8-f15e-446f-a49d-0b4a1f043ac2</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Broken link (202): https://fjedna.shinyapps.io/census-app1/</t>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -679,22 +679,22 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>acd6c43f-6cbd-43c8-9bff-7d9ae6630295</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
+          <t>Invalid Resource URL: https://catalogue.hakai.org/erddap/tabledap/HakaiWaterPropertiesInstrumentProfileProvisional.nc?work_area%2Ccruise%2Chakai_id%2Cvessel%2Coperators%2Ccomments%2Cdevice_model%2Cdevice_sn%2Cdevice_firmware%2Ccast_processing_stage%2Cstation%2Clatitude%2Clongitude%2Cprecise_latitude%2Cprecise_longitude%2Ctime%2Cbottom_date_time%2Cend_date_time%2Cmeasurement_date_time%2Cbottom_depth%2Ctarget_depth%2Cdrop_speed%2Cdirection_flag%2Cdescent_rate%2Cdepth%2Cdepth_UQL%2Cdepth_flag_description%2Cpressure%2Cpressure_UQL%2Cpressure_flag_description%2Cconductivity%2Cconductivity_UQL%2Cconductivity_flag_description%2Ctemperature%2Ctemperature_UQL%2Ctemperature_flag_description%2Csalinity%2Csalinity_UQL%2Csalinity_flag_description%2Cdissolved_oxygen_ml_l%2Cdissolved_oxygen_ml_l_UQL%2Cdissolved_oxygen_ml_l_flag_description%2Crinko_do_ml_l%2Crinko_do_ml_l_UQL%2Crinko_do_ml_l_flag_description%2Cflc%2Cflc_UQL%2Cflc_flag_description%2Cturbidity%2Cturbidity_UQL%2Cturbidity_flag_description%2Cpar%2Cpar_UQL%2Cpar_flag_description%2Cc_star_at%2Cc_star_at_UQL%2Cc_star_at_flag_description%2Cph%2Cph_UQL%2Ccph_flag_description%2Cbackscatter_beta%2Cbackscatter_beta_UQL%2Cbackscatter_beta_flag_description%2Ccdom_ppb%2Ccdom_ppb_UQL%2Ccdom_flag_description&amp;work_area=~%22QUADRA%7CJOHNSTONE%20STRAIT%22&amp;cruise=~%22JS%7CJS%20C%7CJS1%7CJS12%7CJSA1%7CJSA2%7CJSB%7CJSC%7CJSSOCKEYE%7COTHER%2CJSSOCKEYE%7CDI_C%2CDISOCKEYE%7CDI_W%2CDISOCKEYE%7CDISOCKEYE%22 returned status_code=502</t>
         </is>
       </c>
     </row>
@@ -704,42 +704,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>186d3139-66a1-43f9-9ac7-c5607252146e</t>
+          <t>8882a149-fabd-4ecd-98d3-68a2a88aee38</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Metadata mismatch: creator 'Jonathan Bergshoeff' in DataCite not found in CKAN record</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="n">
-        <v>1</v>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>186d3139-66a1-43f9-9ac7-c5607252146e</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: author 'Jon Bergshoeff' in CKAN record not found in DataCite</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="n">
-        <v>0</v>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>acd6c43f-6cbd-43c8-9bff-7d9ae6630295</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Invalid Resource URL: https://catalogue.hakai.org/erddap/tabledap/HakaiWaterPropertiesInstrumentProfileProvisional.nc?work_area%2Ccruise%2Chakai_id%2Cvessel%2Coperators%2Ccomments%2Cdevice_model%2Cdevice_sn%2Cdevice_firmware%2Ccast_processing_stage%2Cstation%2Clatitude%2Clongitude%2Cprecise_latitude%2Cprecise_longitude%2Ctime%2Cbottom_date_time%2Cend_date_time%2Cmeasurement_date_time%2Cbottom_depth%2Ctarget_depth%2Cdrop_speed%2Cdirection_flag%2Cdescent_rate%2Cdepth%2Cdepth_UQL%2Cdepth_flag_description%2Cpressure%2Cpressure_UQL%2Cpressure_flag_description%2Cconductivity%2Cconductivity_UQL%2Cconductivity_flag_description%2Ctemperature%2Ctemperature_UQL%2Ctemperature_flag_description%2Csalinity%2Csalinity_UQL%2Csalinity_flag_description%2Cdissolved_oxygen_ml_l%2Cdissolved_oxygen_ml_l_UQL%2Cdissolved_oxygen_ml_l_flag_description%2Crinko_do_ml_l%2Crinko_do_ml_l_UQL%2Crinko_do_ml_l_flag_description%2Cflc%2Cflc_UQL%2Cflc_flag_description%2Cturbidity%2Cturbidity_UQL%2Cturbidity_flag_description%2Cpar%2Cpar_UQL%2Cpar_flag_description%2Cc_star_at%2Cc_star_at_UQL%2Cc_star_at_flag_description%2Cph%2Cph_UQL%2Ccph_flag_description%2Cbackscatter_beta%2Cbackscatter_beta_UQL%2Cbackscatter_beta_flag_description%2Ccdom_ppb%2Ccdom_ppb_UQL%2Ccdom_flag_description&amp;work_area=~%22QUADRA%7CJOHNSTONE%20STRAIT%22&amp;cruise=~%22JS%7CJS%20C%7CJS1%7CJS12%7CJSA1%7CJSA2%7CJSB%7CJSC%7CJSSOCKEYE%7COTHER%2CJSSOCKEYE%7CDI_C%2CDISOCKEYE%7CDI_W%2CDISOCKEYE%7CDISOCKEYE%22 returned status_code=502</t>
+          <t>Invalid Resource URL: http://docs.turnerdesigns.com/t2/doc/manuals/998-7210.pdf returned status_code=timeout</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deployed 59d2eab0a to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/issues_list.xlsx
+++ b/main/issues_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -449,12 +449,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>30560220-bc44-4020-b424-0abf617d1c00</t>
+          <t>da040f55-984d-490d-b917-a67856de4bac</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Broken link (410): https://coastalmarginsnetwork.org/</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-seastars2024 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -464,12 +464,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>da040f55-984d-490d-b917-a67856de4bac</t>
+          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-seastars2024 returned status_code=404</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -479,12 +479,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
+          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -494,12 +494,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
+          <t>c4932b55-1dd8-4f2f-89da-5822056ecc37</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
+          <t>Broken link (404): https://doi.org/10.21966/ekwk-r335</t>
         </is>
       </c>
     </row>
@@ -509,18 +509,18 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>c4932b55-1dd8-4f2f-89da-5822056ecc37</t>
+          <t>1e13d2ee-580f-4785-838b-908a449781a3</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Broken link (404): https://doi.org/10.21966/ekwk-r335</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -529,22 +529,22 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/GEM-Kit10-repository/tree/main returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>1e13d2ee-580f-4785-838b-908a449781a3</t>
+          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/GEM-Kit10-repository/tree/main returned status_code=404</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -629,12 +629,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
+          <t>c7a168e8-f15e-446f-a49d-0b4a1f043ac2</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Broken link (connection error): https://www2.gov.bc.ca/gov/content/data/geographic-data-services/topographic-data/freshwater</t>
+          <t>Broken link (202): https://fjedna.shinyapps.io/census-app1/</t>
         </is>
       </c>
     </row>
@@ -644,18 +644,18 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>c7a168e8-f15e-446f-a49d-0b4a1f043ac2</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Broken link (202): https://fjedna.shinyapps.io/census-app1/</t>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -664,52 +664,22 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>acd6c43f-6cbd-43c8-9bff-7d9ae6630295</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="n">
-        <v>0</v>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>acd6c43f-6cbd-43c8-9bff-7d9ae6630295</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
           <t>Invalid Resource URL: https://catalogue.hakai.org/erddap/tabledap/HakaiWaterPropertiesInstrumentProfileProvisional.nc?work_area%2Ccruise%2Chakai_id%2Cvessel%2Coperators%2Ccomments%2Cdevice_model%2Cdevice_sn%2Cdevice_firmware%2Ccast_processing_stage%2Cstation%2Clatitude%2Clongitude%2Cprecise_latitude%2Cprecise_longitude%2Ctime%2Cbottom_date_time%2Cend_date_time%2Cmeasurement_date_time%2Cbottom_depth%2Ctarget_depth%2Cdrop_speed%2Cdirection_flag%2Cdescent_rate%2Cdepth%2Cdepth_UQL%2Cdepth_flag_description%2Cpressure%2Cpressure_UQL%2Cpressure_flag_description%2Cconductivity%2Cconductivity_UQL%2Cconductivity_flag_description%2Ctemperature%2Ctemperature_UQL%2Ctemperature_flag_description%2Csalinity%2Csalinity_UQL%2Csalinity_flag_description%2Cdissolved_oxygen_ml_l%2Cdissolved_oxygen_ml_l_UQL%2Cdissolved_oxygen_ml_l_flag_description%2Crinko_do_ml_l%2Crinko_do_ml_l_UQL%2Crinko_do_ml_l_flag_description%2Cflc%2Cflc_UQL%2Cflc_flag_description%2Cturbidity%2Cturbidity_UQL%2Cturbidity_flag_description%2Cpar%2Cpar_UQL%2Cpar_flag_description%2Cc_star_at%2Cc_star_at_UQL%2Cc_star_at_flag_description%2Cph%2Cph_UQL%2Ccph_flag_description%2Cbackscatter_beta%2Cbackscatter_beta_UQL%2Cbackscatter_beta_flag_description%2Ccdom_ppb%2Ccdom_ppb_UQL%2Ccdom_flag_description&amp;work_area=~%22QUADRA%7CJOHNSTONE%20STRAIT%22&amp;cruise=~%22JS%7CJS%20C%7CJS1%7CJS12%7CJSA1%7CJSA2%7CJSB%7CJSC%7CJSSOCKEYE%7COTHER%2CJSSOCKEYE%7CDI_C%2CDISOCKEYE%7CDI_W%2CDISOCKEYE%7CDISOCKEYE%22 returned status_code=502</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="n">
-        <v>0</v>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>8882a149-fabd-4ecd-98d3-68a2a88aee38</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Invalid Resource URL: http://docs.turnerdesigns.com/t2/doc/manuals/998-7210.pdf returned status_code=timeout</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deployed fc5854078 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/issues_list.xlsx
+++ b/main/issues_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -434,12 +434,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>bd461764-55b0-4c63-935a-5e9d1d5a6fed</t>
+          <t>bf7c05e8-510d-4449-9e81-4c358ff3f440</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-itracksept2023 returned status_code=404</t>
+          <t>Broken link (connection error): http://docs.turnerdesigns.com/t2/doc/manuals/998-7210.pdf</t>
         </is>
       </c>
     </row>
@@ -449,12 +449,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>da040f55-984d-490d-b917-a67856de4bac</t>
+          <t>bd461764-55b0-4c63-935a-5e9d1d5a6fed</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-seastars2024 returned status_code=404</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-itracksept2023 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -464,12 +464,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
+          <t>30560220-bc44-4020-b424-0abf617d1c00</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
+          <t>Broken link (410): https://coastalmarginsnetwork.org/</t>
         </is>
       </c>
     </row>
@@ -479,12 +479,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
+          <t>da040f55-984d-490d-b917-a67856de4bac</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-seastars2024 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -494,12 +494,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>c4932b55-1dd8-4f2f-89da-5822056ecc37</t>
+          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Broken link (404): https://doi.org/10.21966/ekwk-r335</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -509,27 +509,27 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>1e13d2ee-580f-4785-838b-908a449781a3</t>
+          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>1e13d2ee-580f-4785-838b-908a449781a3</t>
+          <t>c4932b55-1dd8-4f2f-89da-5822056ecc37</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/GEM-Kit10-repository/tree/main returned status_code=404</t>
+          <t>Broken link (404): https://doi.org/10.21966/ekwk-r335</t>
         </is>
       </c>
     </row>
@@ -539,27 +539,27 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
+          <t>1e13d2ee-580f-4785-838b-908a449781a3</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
+          <t>1e13d2ee-580f-4785-838b-908a449781a3</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-qu5-mooring-data</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/GEM-Kit10-repository/tree/main returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -569,12 +569,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
+          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -584,12 +584,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
+          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
+          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-qu5-mooring-data</t>
         </is>
       </c>
     </row>
@@ -599,27 +599,27 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -629,42 +629,42 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>c7a168e8-f15e-446f-a49d-0b4a1f043ac2</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Broken link (202): https://fjedna.shinyapps.io/census-app1/</t>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>c7a168e8-f15e-446f-a49d-0b4a1f043ac2</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
+          <t>Broken link (202): https://fjedna.shinyapps.io/census-app1/</t>
         </is>
       </c>
     </row>
@@ -674,10 +674,70 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>1</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>0</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>186d3139-66a1-43f9-9ac7-c5607252146e</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Metadata mismatch: version CKAN='1.1' | DataCite='1.0'</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>0</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>9cdf1117-a07a-4fc1-ba03-e69f3e2963fb</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Broken link (404): https://doi.org/10.21966/ekwk-r335</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>0</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
           <t>acd6c43f-6cbd-43c8-9bff-7d9ae6630295</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>Invalid Resource URL: https://catalogue.hakai.org/erddap/tabledap/HakaiWaterPropertiesInstrumentProfileProvisional.nc?work_area%2Ccruise%2Chakai_id%2Cvessel%2Coperators%2Ccomments%2Cdevice_model%2Cdevice_sn%2Cdevice_firmware%2Ccast_processing_stage%2Cstation%2Clatitude%2Clongitude%2Cprecise_latitude%2Cprecise_longitude%2Ctime%2Cbottom_date_time%2Cend_date_time%2Cmeasurement_date_time%2Cbottom_depth%2Ctarget_depth%2Cdrop_speed%2Cdirection_flag%2Cdescent_rate%2Cdepth%2Cdepth_UQL%2Cdepth_flag_description%2Cpressure%2Cpressure_UQL%2Cpressure_flag_description%2Cconductivity%2Cconductivity_UQL%2Cconductivity_flag_description%2Ctemperature%2Ctemperature_UQL%2Ctemperature_flag_description%2Csalinity%2Csalinity_UQL%2Csalinity_flag_description%2Cdissolved_oxygen_ml_l%2Cdissolved_oxygen_ml_l_UQL%2Cdissolved_oxygen_ml_l_flag_description%2Crinko_do_ml_l%2Crinko_do_ml_l_UQL%2Crinko_do_ml_l_flag_description%2Cflc%2Cflc_UQL%2Cflc_flag_description%2Cturbidity%2Cturbidity_UQL%2Cturbidity_flag_description%2Cpar%2Cpar_UQL%2Cpar_flag_description%2Cc_star_at%2Cc_star_at_UQL%2Cc_star_at_flag_description%2Cph%2Cph_UQL%2Ccph_flag_description%2Cbackscatter_beta%2Cbackscatter_beta_UQL%2Cbackscatter_beta_flag_description%2Ccdom_ppb%2Ccdom_ppb_UQL%2Ccdom_flag_description&amp;work_area=~%22QUADRA%7CJOHNSTONE%20STRAIT%22&amp;cruise=~%22JS%7CJS%20C%7CJS1%7CJS12%7CJSA1%7CJSA2%7CJSB%7CJSC%7CJSSOCKEYE%7COTHER%2CJSSOCKEYE%7CDI_C%2CDISOCKEYE%7CDI_W%2CDISOCKEYE%7CDISOCKEYE%22 returned status_code=502</t>
         </is>

</xml_diff>

<commit_message>
Deployed 572e1d565 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/issues_list.xlsx
+++ b/main/issues_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -674,18 +674,18 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+          <t>Record DOI HTTPS link is failling: https://doi.org/10.21966/abh1-kk96 status_code=502</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -694,22 +694,22 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>186d3139-66a1-43f9-9ac7-c5607252146e</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Metadata mismatch: version CKAN='1.1' | DataCite='1.0'</t>
+          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
         </is>
       </c>
     </row>
@@ -719,25 +719,55 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>9cdf1117-a07a-4fc1-ba03-e69f3e2963fb</t>
+          <t>a3b64e3a-3315-4d64-81d8-6e772e44951d</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Broken link (404): https://doi.org/10.21966/ekwk-r335</t>
+          <t>Tentative dataset should not have a version</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
+          <t>a3b64e3a-3315-4d64-81d8-6e772e44951d</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Broken link (404): https://doi.org/10.21966/ekwk-r335</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>0</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>9cdf1117-a07a-4fc1-ba03-e69f3e2963fb</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Broken link (404): https://doi.org/10.21966/ekwk-r335</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>0</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
           <t>acd6c43f-6cbd-43c8-9bff-7d9ae6630295</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>Invalid Resource URL: https://catalogue.hakai.org/erddap/tabledap/HakaiWaterPropertiesInstrumentProfileProvisional.nc?work_area%2Ccruise%2Chakai_id%2Cvessel%2Coperators%2Ccomments%2Cdevice_model%2Cdevice_sn%2Cdevice_firmware%2Ccast_processing_stage%2Cstation%2Clatitude%2Clongitude%2Cprecise_latitude%2Cprecise_longitude%2Ctime%2Cbottom_date_time%2Cend_date_time%2Cmeasurement_date_time%2Cbottom_depth%2Ctarget_depth%2Cdrop_speed%2Cdirection_flag%2Cdescent_rate%2Cdepth%2Cdepth_UQL%2Cdepth_flag_description%2Cpressure%2Cpressure_UQL%2Cpressure_flag_description%2Cconductivity%2Cconductivity_UQL%2Cconductivity_flag_description%2Ctemperature%2Ctemperature_UQL%2Ctemperature_flag_description%2Csalinity%2Csalinity_UQL%2Csalinity_flag_description%2Cdissolved_oxygen_ml_l%2Cdissolved_oxygen_ml_l_UQL%2Cdissolved_oxygen_ml_l_flag_description%2Crinko_do_ml_l%2Crinko_do_ml_l_UQL%2Crinko_do_ml_l_flag_description%2Cflc%2Cflc_UQL%2Cflc_flag_description%2Cturbidity%2Cturbidity_UQL%2Cturbidity_flag_description%2Cpar%2Cpar_UQL%2Cpar_flag_description%2Cc_star_at%2Cc_star_at_UQL%2Cc_star_at_flag_description%2Cph%2Cph_UQL%2Ccph_flag_description%2Cbackscatter_beta%2Cbackscatter_beta_UQL%2Cbackscatter_beta_flag_description%2Ccdom_ppb%2Ccdom_ppb_UQL%2Ccdom_flag_description&amp;work_area=~%22QUADRA%7CJOHNSTONE%20STRAIT%22&amp;cruise=~%22JS%7CJS%20C%7CJS1%7CJS12%7CJSA1%7CJSA2%7CJSB%7CJSC%7CJSSOCKEYE%7COTHER%2CJSSOCKEYE%7CDI_C%2CDISOCKEYE%7CDI_W%2CDISOCKEYE%7CDISOCKEYE%22 returned status_code=502</t>
         </is>

</xml_diff>

<commit_message>
Deployed 25b9f3853 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/issues_list.xlsx
+++ b/main/issues_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -445,16 +445,16 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>bd461764-55b0-4c63-935a-5e9d1d5a6fed</t>
+          <t>bf7c05e8-510d-4449-9e81-4c358ff3f440</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-itracksept2023 returned status_code=404</t>
+          <t>Metadata mismatch: related identifier 'https://catalogue.hakai.org/dataset/ca-cioos_a8f45d4f-6e6b-4cce-a92d-28e8924148b7' (IsPartOf) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -464,12 +464,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>30560220-bc44-4020-b424-0abf617d1c00</t>
+          <t>bd461764-55b0-4c63-935a-5e9d1d5a6fed</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Broken link (410): https://coastalmarginsnetwork.org/</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-itracksept2023 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -479,12 +479,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>da040f55-984d-490d-b917-a67856de4bac</t>
+          <t>30560220-bc44-4020-b424-0abf617d1c00</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-seastars2024 returned status_code=404</t>
+          <t>Broken link (410): https://coastalmarginsnetwork.org/</t>
         </is>
       </c>
     </row>
@@ -494,12 +494,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
+          <t>da040f55-984d-490d-b917-a67856de4bac</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-seastars2024 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -509,12 +509,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
+          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -524,42 +524,42 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>c4932b55-1dd8-4f2f-89da-5822056ecc37</t>
+          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Broken link (404): https://doi.org/10.21966/ekwk-r335</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>1e13d2ee-580f-4785-838b-908a449781a3</t>
+          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Metadata mismatch: related identifier 'https://catalogue.hakai.org/dataset/ca-cioos_a8f45d4f-6e6b-4cce-a92d-28e8924148b7' (IsPartOf) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>1e13d2ee-580f-4785-838b-908a449781a3</t>
+          <t>c4932b55-1dd8-4f2f-89da-5822056ecc37</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/GEM-Kit10-repository/tree/main returned status_code=404</t>
+          <t>Broken link (404): https://doi.org/10.21966/ekwk-r335</t>
         </is>
       </c>
     </row>
@@ -569,27 +569,27 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
+          <t>1e13d2ee-580f-4785-838b-908a449781a3</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
+          <t>1e13d2ee-580f-4785-838b-908a449781a3</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-qu5-mooring-data</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/GEM-Kit10-repository/tree/main returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -599,12 +599,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
+          <t>5042c858-d375-42f5-82e0-ee1e4da962b6</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
+          <t>Metadata mismatch: related identifier 'https://catalogue.hakai.org/dataset/ca-cioos_a8f45d4f-6e6b-4cce-a92d-28e8924148b7' (IsPartOf) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -614,12 +614,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
+          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -629,27 +629,27 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-qu5-mooring-data</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>d3ed88cb-4f38-4c2e-a966-3dd49c9cafec</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
+          <t>Metadata mismatch: related identifier 'https://catalogue.hakai.org/dataset/ca-cioos_a8f45d4f-6e6b-4cce-a92d-28e8924148b7' (IsPartOf) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -659,12 +659,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>c7a168e8-f15e-446f-a49d-0b4a1f043ac2</t>
+          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Broken link (202): https://fjedna.shinyapps.io/census-app1/</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -674,12 +674,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>d3c4dde5-38b2-480d-a4e7-228bde9eb537</t>
+          <t>cb0f4710-d78a-4073-959c-95f874f88711</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Record DOI HTTPS link is failling: https://doi.org/10.21966/abh1-kk96 status_code=502</t>
+          <t>Metadata mismatch: related identifier 'https://catalogue.hakai.org/dataset/ca-cioos_a8f45d4f-6e6b-4cce-a92d-28e8924148b7' (IsPartOf) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -689,57 +689,57 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>a3b64e3a-3315-4d64-81d8-6e772e44951d</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Tentative dataset should not have a version</t>
+          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>a3b64e3a-3315-4d64-81d8-6e772e44951d</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Broken link (404): https://doi.org/10.21966/ekwk-r335</t>
+          <t>Metadata mismatch: related identifier 'https://catalogue.hakai.org/dataset/ca-cioos_a8f45d4f-6e6b-4cce-a92d-28e8924148b7' (IsPartOf) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
@@ -749,12 +749,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>9cdf1117-a07a-4fc1-ba03-e69f3e2963fb</t>
+          <t>c7a168e8-f15e-446f-a49d-0b4a1f043ac2</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Broken link (404): https://doi.org/10.21966/ekwk-r335</t>
+          <t>Broken link (202): https://fjedna.shinyapps.io/census-app1/</t>
         </is>
       </c>
     </row>
@@ -764,10 +764,130 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>1</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>2</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Metadata mismatch: related identifier 'https://catalogue.hakai.org/dataset/ca-cioos_a8f45d4f-6e6b-4cce-a92d-28e8924148b7' (IsPartOf) in DataCite not found in CKAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>0</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>a3b64e3a-3315-4d64-81d8-6e772e44951d</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Tentative dataset should not have a version</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>1</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>a3b64e3a-3315-4d64-81d8-6e772e44951d</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Broken link (404): https://doi.org/10.21966/ekwk-r335</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>0</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>186d3139-66a1-43f9-9ac7-c5607252146e</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Metadata mismatch: related identifier 'https://catalogue.hakai.org/dataset/ca-cioos_a8f45d4f-6e6b-4cce-a92d-28e8924148b7' (IsPartOf) in DataCite not found in CKAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>0</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>3fbbd892-55cd-4c96-9669-cecefe726b3f</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Metadata mismatch: related identifier 'https://catalogue.hakai.org/dataset/ca-cioos_a8f45d4f-6e6b-4cce-a92d-28e8924148b7' (IsPartOf) in DataCite not found in CKAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>0</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>9cdf1117-a07a-4fc1-ba03-e69f3e2963fb</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Broken link (404): https://doi.org/10.21966/ekwk-r335</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>0</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
           <t>acd6c43f-6cbd-43c8-9bff-7d9ae6630295</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>Invalid Resource URL: https://catalogue.hakai.org/erddap/tabledap/HakaiWaterPropertiesInstrumentProfileProvisional.nc?work_area%2Ccruise%2Chakai_id%2Cvessel%2Coperators%2Ccomments%2Cdevice_model%2Cdevice_sn%2Cdevice_firmware%2Ccast_processing_stage%2Cstation%2Clatitude%2Clongitude%2Cprecise_latitude%2Cprecise_longitude%2Ctime%2Cbottom_date_time%2Cend_date_time%2Cmeasurement_date_time%2Cbottom_depth%2Ctarget_depth%2Cdrop_speed%2Cdirection_flag%2Cdescent_rate%2Cdepth%2Cdepth_UQL%2Cdepth_flag_description%2Cpressure%2Cpressure_UQL%2Cpressure_flag_description%2Cconductivity%2Cconductivity_UQL%2Cconductivity_flag_description%2Ctemperature%2Ctemperature_UQL%2Ctemperature_flag_description%2Csalinity%2Csalinity_UQL%2Csalinity_flag_description%2Cdissolved_oxygen_ml_l%2Cdissolved_oxygen_ml_l_UQL%2Cdissolved_oxygen_ml_l_flag_description%2Crinko_do_ml_l%2Crinko_do_ml_l_UQL%2Crinko_do_ml_l_flag_description%2Cflc%2Cflc_UQL%2Cflc_flag_description%2Cturbidity%2Cturbidity_UQL%2Cturbidity_flag_description%2Cpar%2Cpar_UQL%2Cpar_flag_description%2Cc_star_at%2Cc_star_at_UQL%2Cc_star_at_flag_description%2Cph%2Cph_UQL%2Ccph_flag_description%2Cbackscatter_beta%2Cbackscatter_beta_UQL%2Cbackscatter_beta_flag_description%2Ccdom_ppb%2Ccdom_ppb_UQL%2Ccdom_flag_description&amp;work_area=~%22QUADRA%7CJOHNSTONE%20STRAIT%22&amp;cruise=~%22JS%7CJS%20C%7CJS1%7CJS12%7CJSA1%7CJSA2%7CJSB%7CJSC%7CJSSOCKEYE%7COTHER%2CJSSOCKEYE%7CDI_C%2CDISOCKEYE%7CDI_W%2CDISOCKEYE%7CDISOCKEYE%22 returned status_code=502</t>
         </is>

</xml_diff>

<commit_message>
Deployed 6191c3393 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/issues_list.xlsx
+++ b/main/issues_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C32"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -434,27 +434,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>bf7c05e8-510d-4449-9e81-4c358ff3f440</t>
+          <t>bd461764-55b0-4c63-935a-5e9d1d5a6fed</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Broken link (connection error): http://docs.turnerdesigns.com/t2/doc/manuals/998-7210.pdf</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-itracksept2023 returned status_code=404</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>bf7c05e8-510d-4449-9e81-4c358ff3f440</t>
+          <t>30560220-bc44-4020-b424-0abf617d1c00</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://catalogue.hakai.org/dataset/ca-cioos_a8f45d4f-6e6b-4cce-a92d-28e8924148b7' (IsPartOf) in DataCite not found in CKAN</t>
+          <t>Broken link (410): https://coastalmarginsnetwork.org/</t>
         </is>
       </c>
     </row>
@@ -464,12 +464,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>bd461764-55b0-4c63-935a-5e9d1d5a6fed</t>
+          <t>da040f55-984d-490d-b917-a67856de4bac</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-itracksept2023 returned status_code=404</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-seastars2024 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -479,12 +479,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>30560220-bc44-4020-b424-0abf617d1c00</t>
+          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Broken link (410): https://coastalmarginsnetwork.org/</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -494,12 +494,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>da040f55-984d-490d-b917-a67856de4bac</t>
+          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-seastars2024 returned status_code=404</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -509,12 +509,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>f409100d-95e4-4933-a927-fdf8d3b83204</t>
+          <t>c4932b55-1dd8-4f2f-89da-5822056ecc37</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=12Spn0fnOC91dLOahgcf94_lrELHvXFX6 returned status_code=404</t>
+          <t>Broken link (404): https://doi.org/10.21966/ekwk-r335</t>
         </is>
       </c>
     </row>
@@ -524,12 +524,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
+          <t>1e13d2ee-580f-4785-838b-908a449781a3</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-zooplankton-microscopy-dataset returned status_code=404</t>
+          <t>No funder</t>
         </is>
       </c>
     </row>
@@ -539,12 +539,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>139df6dd-772b-424f-b830-30a5ba6abfc6</t>
+          <t>1e13d2ee-580f-4785-838b-908a449781a3</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://catalogue.hakai.org/dataset/ca-cioos_a8f45d4f-6e6b-4cce-a92d-28e8924148b7' (IsPartOf) in DataCite not found in CKAN</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/GEM-Kit10-repository/tree/main returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -554,12 +554,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>c4932b55-1dd8-4f2f-89da-5822056ecc37</t>
+          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Broken link (404): https://doi.org/10.21966/ekwk-r335</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -569,27 +569,27 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>1e13d2ee-580f-4785-838b-908a449781a3</t>
+          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>No funder</t>
+          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-qu5-mooring-data</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>1e13d2ee-580f-4785-838b-908a449781a3</t>
+          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/GEM-Kit10-repository/tree/main returned status_code=404</t>
+          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -599,12 +599,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>5042c858-d375-42f5-82e0-ee1e4da962b6</t>
+          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://catalogue.hakai.org/dataset/ca-cioos_a8f45d4f-6e6b-4cce-a92d-28e8924148b7' (IsPartOf) in DataCite not found in CKAN</t>
+          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
         </is>
       </c>
     </row>
@@ -614,27 +614,27 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>e4038a43-060b-474e-b6f2-ea68d0081053</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/hakai-wetlab-calliarthron2023 returned status_code=404</t>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>7c2b8668-75a3-4fc8-bff3-bdae5d95f52d</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Broken link (404): https://github.com/HakaiInstitute/hakai-qu5-mooring-data</t>
+          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
         </is>
       </c>
     </row>
@@ -644,12 +644,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>d3ed88cb-4f38-4c2e-a966-3dd49c9cafec</t>
+          <t>c7a168e8-f15e-446f-a49d-0b4a1f043ac2</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://catalogue.hakai.org/dataset/ca-cioos_a8f45d4f-6e6b-4cce-a92d-28e8924148b7' (IsPartOf) in DataCite not found in CKAN</t>
+          <t>Broken link (202): https://fjedna.shinyapps.io/census-app1/</t>
         </is>
       </c>
     </row>
@@ -659,12 +659,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>0e92249d-74e1-4253-a8a5-876d08a8ff65</t>
+          <t>a3b64e3a-3315-4d64-81d8-6e772e44951d</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://github.com/HakaiInstitute/Biogeochemical-Sampling-of-28-Streams-on-Vancouver-Island returned status_code=404</t>
+          <t>Broken link (404): https://doi.org/10.21966/ekwk-r335</t>
         </is>
       </c>
     </row>
@@ -674,27 +674,27 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>cb0f4710-d78a-4073-959c-95f874f88711</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Metadata mismatch: related identifier 'https://catalogue.hakai.org/dataset/ca-cioos_a8f45d4f-6e6b-4cce-a92d-28e8924148b7' (IsPartOf) in DataCite not found in CKAN</t>
+          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>def2a409-2319-4e8c-a584-9a467f044ada</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Invalid Resource URL: https://drive.google.com/open?id=0B3dfJwMwT2k4RzNYOGFUcFNpUms returned status_code=404</t>
+          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
         </is>
       </c>
     </row>
@@ -704,190 +704,40 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>186d3139-66a1-43f9-9ac7-c5607252146e</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
+          <t>Metadata mismatch: related identifier 'https://catalogue.hakai.org/dataset/ca-cioos_a8f45d4f-6e6b-4cce-a92d-28e8924148b7' (IsPartOf) in DataCite not found in CKAN</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>9cdf1117-a07a-4fc1-ba03-e69f3e2963fb</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
+          <t>Broken link (404): https://doi.org/10.21966/ekwk-r335</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>acd6c43f-6cbd-43c8-9bff-7d9ae6630295</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: related identifier 'https://catalogue.hakai.org/dataset/ca-cioos_a8f45d4f-6e6b-4cce-a92d-28e8924148b7' (IsPartOf) in DataCite not found in CKAN</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="n">
-        <v>0</v>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>c7a168e8-f15e-446f-a49d-0b4a1f043ac2</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Broken link (202): https://fjedna.shinyapps.io/census-app1/</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="n">
-        <v>0</v>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Broken link (202): https://doi.org/10.1109/IGARSS.2012.6351194</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="n">
-        <v>1</v>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Broken link (202): https://doi.org/10.1109/PACRIM47961.2019.8985053</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="n">
-        <v>2</v>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: related identifier 'https://catalogue.hakai.org/dataset/ca-cioos_a8f45d4f-6e6b-4cce-a92d-28e8924148b7' (IsPartOf) in DataCite not found in CKAN</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="n">
-        <v>0</v>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>a3b64e3a-3315-4d64-81d8-6e772e44951d</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Tentative dataset should not have a version</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="n">
-        <v>1</v>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>a3b64e3a-3315-4d64-81d8-6e772e44951d</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>Broken link (404): https://doi.org/10.21966/ekwk-r335</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="n">
-        <v>0</v>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>186d3139-66a1-43f9-9ac7-c5607252146e</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: related identifier 'https://catalogue.hakai.org/dataset/ca-cioos_a8f45d4f-6e6b-4cce-a92d-28e8924148b7' (IsPartOf) in DataCite not found in CKAN</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="n">
-        <v>0</v>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>3fbbd892-55cd-4c96-9669-cecefe726b3f</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Metadata mismatch: related identifier 'https://catalogue.hakai.org/dataset/ca-cioos_a8f45d4f-6e6b-4cce-a92d-28e8924148b7' (IsPartOf) in DataCite not found in CKAN</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="n">
-        <v>0</v>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>9cdf1117-a07a-4fc1-ba03-e69f3e2963fb</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>Broken link (404): https://doi.org/10.21966/ekwk-r335</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="n">
-        <v>0</v>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>acd6c43f-6cbd-43c8-9bff-7d9ae6630295</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
         <is>
           <t>Invalid Resource URL: https://catalogue.hakai.org/erddap/tabledap/HakaiWaterPropertiesInstrumentProfileProvisional.nc?work_area%2Ccruise%2Chakai_id%2Cvessel%2Coperators%2Ccomments%2Cdevice_model%2Cdevice_sn%2Cdevice_firmware%2Ccast_processing_stage%2Cstation%2Clatitude%2Clongitude%2Cprecise_latitude%2Cprecise_longitude%2Ctime%2Cbottom_date_time%2Cend_date_time%2Cmeasurement_date_time%2Cbottom_depth%2Ctarget_depth%2Cdrop_speed%2Cdirection_flag%2Cdescent_rate%2Cdepth%2Cdepth_UQL%2Cdepth_flag_description%2Cpressure%2Cpressure_UQL%2Cpressure_flag_description%2Cconductivity%2Cconductivity_UQL%2Cconductivity_flag_description%2Ctemperature%2Ctemperature_UQL%2Ctemperature_flag_description%2Csalinity%2Csalinity_UQL%2Csalinity_flag_description%2Cdissolved_oxygen_ml_l%2Cdissolved_oxygen_ml_l_UQL%2Cdissolved_oxygen_ml_l_flag_description%2Crinko_do_ml_l%2Crinko_do_ml_l_UQL%2Crinko_do_ml_l_flag_description%2Cflc%2Cflc_UQL%2Cflc_flag_description%2Cturbidity%2Cturbidity_UQL%2Cturbidity_flag_description%2Cpar%2Cpar_UQL%2Cpar_flag_description%2Cc_star_at%2Cc_star_at_UQL%2Cc_star_at_flag_description%2Cph%2Cph_UQL%2Ccph_flag_description%2Cbackscatter_beta%2Cbackscatter_beta_UQL%2Cbackscatter_beta_flag_description%2Ccdom_ppb%2Ccdom_ppb_UQL%2Ccdom_flag_description&amp;work_area=~%22QUADRA%7CJOHNSTONE%20STRAIT%22&amp;cruise=~%22JS%7CJS%20C%7CJS1%7CJS12%7CJSA1%7CJSA2%7CJSB%7CJSC%7CJSSOCKEYE%7COTHER%2CJSSOCKEYE%7CDI_C%2CDISOCKEYE%7CDI_W%2CDISOCKEYE%7CDISOCKEYE%22 returned status_code=502</t>
         </is>

</xml_diff>